<commit_message>
big upgrade for miss pattern, strokes gained category and new UI
</commit_message>
<xml_diff>
--- a/SG_baseline.xlsx
+++ b/SG_baseline.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\NikolaiAasprong\golf-stats\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9AD5015-85AB-4ABB-84FE-C0E1EEF802CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E11CE72C-572D-49FC-8061-1D20AEDF0125}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{B64AB023-654D-4F45-8500-8FC89343C9DD}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{B64AB023-654D-4F45-8500-8FC89343C9DD}"/>
   </bookViews>
   <sheets>
     <sheet name="source" sheetId="1" r:id="rId1"/>
@@ -37,8 +37,30 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="16">
   <si>
     <t>DISTANCE</t>
   </si>
@@ -85,19 +107,7 @@
     <t>AVG SHORT GAME</t>
   </si>
   <si>
-    <t>Expected shots</t>
-  </si>
-  <si>
-    <t>Tee shot distance [m]</t>
-  </si>
-  <si>
-    <t>Approach shot distance [m]</t>
-  </si>
-  <si>
-    <t>Short game distance [m]</t>
-  </si>
-  <si>
-    <t>Putting distance [m]</t>
+    <t>manually created</t>
   </si>
 </sst>
 </file>
@@ -105,8 +115,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="167" formatCode="0.00000"/>
-    <numFmt numFmtId="168" formatCode="0.0000"/>
+    <numFmt numFmtId="164" formatCode="0.00000"/>
+    <numFmt numFmtId="165" formatCode="0.0000"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -136,7 +146,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -149,8 +159,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="12">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -233,77 +249,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -338,14 +288,11 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2171,7 +2118,7 @@
     <col min="12" max="12" width="14.7109375" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="16.42578125" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="16.42578125" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="15.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2242,9 +2189,8 @@
         <f>source!A2/metric!$W$2</f>
         <v>9.1439999861011216</v>
       </c>
-      <c r="B2">
-        <f>source!B2</f>
-        <v>0</v>
+      <c r="B2" s="14">
+        <v>2.74</v>
       </c>
       <c r="C2">
         <f>source!C2</f>
@@ -2258,9 +2204,8 @@
         <f>source!E2</f>
         <v>2.41</v>
       </c>
-      <c r="F2">
-        <f>source!F2</f>
-        <v>0</v>
+      <c r="F2" s="14">
+        <v>3.5</v>
       </c>
       <c r="I2">
         <f>source!I2/metric!$V$2</f>
@@ -2306,9 +2251,8 @@
         <f>source!A3/metric!$W$2</f>
         <v>13.715999979151681</v>
       </c>
-      <c r="B3">
-        <f>source!B3</f>
-        <v>0</v>
+      <c r="B3" s="14">
+        <v>2.75</v>
       </c>
       <c r="C3">
         <f>source!C3</f>
@@ -2322,9 +2266,8 @@
         <f>source!E3</f>
         <v>2.4700000000000002</v>
       </c>
-      <c r="F3">
-        <f>source!F3</f>
-        <v>0</v>
+      <c r="F3" s="14">
+        <v>3.5</v>
       </c>
       <c r="I3">
         <f>source!I3/metric!$V$2</f>
@@ -2364,9 +2307,8 @@
         <f>source!A4/metric!$W$2</f>
         <v>18.287999972202243</v>
       </c>
-      <c r="B4">
-        <f>source!B4</f>
-        <v>0</v>
+      <c r="B4" s="14">
+        <v>2.76</v>
       </c>
       <c r="C4">
         <f>source!C4</f>
@@ -2380,9 +2322,8 @@
         <f>source!E4</f>
         <v>2.5299999999999998</v>
       </c>
-      <c r="F4">
-        <f>source!F4</f>
-        <v>0</v>
+      <c r="F4" s="14">
+        <v>3.5</v>
       </c>
       <c r="I4">
         <f>source!I4/metric!$V$2</f>
@@ -2422,9 +2363,8 @@
         <f>source!A5/metric!$W$2</f>
         <v>22.859999965252801</v>
       </c>
-      <c r="B5">
-        <f>source!B5</f>
-        <v>0</v>
+      <c r="B5" s="14">
+        <v>2.77</v>
       </c>
       <c r="C5">
         <f>source!C5</f>
@@ -2438,9 +2378,8 @@
         <f>source!E5</f>
         <v>2.59</v>
       </c>
-      <c r="F5">
-        <f>source!F5</f>
-        <v>0</v>
+      <c r="F5" s="14">
+        <v>3.55</v>
       </c>
       <c r="I5">
         <f>source!I5/metric!$V$2</f>
@@ -2480,9 +2419,8 @@
         <f>source!A6/metric!$W$2</f>
         <v>27.431999958303361</v>
       </c>
-      <c r="B6">
-        <f>source!B6</f>
-        <v>0</v>
+      <c r="B6" s="14">
+        <v>2.78</v>
       </c>
       <c r="C6">
         <f>source!C6</f>
@@ -2496,9 +2434,8 @@
         <f>source!E6</f>
         <v>2.67</v>
       </c>
-      <c r="F6">
-        <f>source!F6</f>
-        <v>0</v>
+      <c r="F6" s="14">
+        <v>3.55</v>
       </c>
       <c r="I6">
         <f>source!I6/metric!$V$2</f>
@@ -2538,9 +2475,8 @@
         <f>source!A7/metric!$W$2</f>
         <v>32.003999951353926</v>
       </c>
-      <c r="B7">
-        <f>source!B7</f>
-        <v>0</v>
+      <c r="B7" s="14">
+        <v>2.79</v>
       </c>
       <c r="C7">
         <f>source!C7</f>
@@ -2554,9 +2490,8 @@
         <f>source!E7</f>
         <v>2.76</v>
       </c>
-      <c r="F7">
-        <f>source!F7</f>
-        <v>0</v>
+      <c r="F7" s="14">
+        <v>3.55</v>
       </c>
       <c r="I7">
         <f>source!I7/metric!$V$2</f>
@@ -2596,9 +2531,8 @@
         <f>source!A8/metric!$W$2</f>
         <v>36.575999944404487</v>
       </c>
-      <c r="B8">
-        <f>source!B8</f>
-        <v>0</v>
+      <c r="B8" s="14">
+        <v>2.8</v>
       </c>
       <c r="C8">
         <f>source!C8</f>
@@ -2612,9 +2546,8 @@
         <f>source!E8</f>
         <v>2.82</v>
       </c>
-      <c r="F8">
-        <f>source!F8</f>
-        <v>0</v>
+      <c r="F8" s="14">
+        <v>3.6</v>
       </c>
       <c r="I8">
         <f>source!I8/metric!$V$2</f>
@@ -2634,9 +2567,8 @@
         <f>source!A9/metric!$W$2</f>
         <v>41.147999937455047</v>
       </c>
-      <c r="B9">
-        <f>source!B9</f>
-        <v>0</v>
+      <c r="B9" s="14">
+        <v>2.81</v>
       </c>
       <c r="C9">
         <f>source!C9</f>
@@ -2650,9 +2582,8 @@
         <f>source!E9</f>
         <v>2.9</v>
       </c>
-      <c r="F9">
-        <f>source!F9</f>
-        <v>0</v>
+      <c r="F9" s="14">
+        <v>3.6</v>
       </c>
       <c r="I9">
         <f>source!I9/metric!$V$2</f>
@@ -2665,6 +2596,9 @@
       <c r="M9" s="12">
         <f t="shared" si="0"/>
         <v>2.78</v>
+      </c>
+      <c r="V9" s="14" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="10" spans="1:23" x14ac:dyDescent="0.25">
@@ -2672,9 +2606,8 @@
         <f>source!A10/metric!$W$2</f>
         <v>45.719999930505601</v>
       </c>
-      <c r="B10">
-        <f>source!B10</f>
-        <v>0</v>
+      <c r="B10" s="14">
+        <v>2.82</v>
       </c>
       <c r="C10">
         <f>source!C10</f>
@@ -2688,9 +2621,8 @@
         <f>source!E10</f>
         <v>2.98</v>
       </c>
-      <c r="F10">
-        <f>source!F10</f>
-        <v>0</v>
+      <c r="F10" s="14">
+        <v>3.6</v>
       </c>
       <c r="I10">
         <f>source!I10/metric!$V$2</f>
@@ -2710,9 +2642,8 @@
         <f>source!A11/metric!$W$2</f>
         <v>50.291999923556162</v>
       </c>
-      <c r="B11">
-        <f>source!B11</f>
-        <v>0</v>
+      <c r="B11" s="14">
+        <v>2.83</v>
       </c>
       <c r="C11">
         <f>source!C11</f>
@@ -2726,9 +2657,8 @@
         <f>source!E11</f>
         <v>3.07</v>
       </c>
-      <c r="F11">
-        <f>source!F11</f>
-        <v>0</v>
+      <c r="F11" s="14">
+        <v>3.65</v>
       </c>
       <c r="I11">
         <f>source!I11/metric!$V$2</f>
@@ -2748,9 +2678,8 @@
         <f>source!A12/metric!$W$2</f>
         <v>54.863999916606723</v>
       </c>
-      <c r="B12">
-        <f>source!B12</f>
-        <v>0</v>
+      <c r="B12" s="14">
+        <v>2.84</v>
       </c>
       <c r="C12">
         <f>source!C12</f>
@@ -2764,9 +2693,8 @@
         <f>source!E12</f>
         <v>3.15</v>
       </c>
-      <c r="F12">
-        <f>source!F12</f>
-        <v>0</v>
+      <c r="F12" s="14">
+        <v>3.65</v>
       </c>
       <c r="I12">
         <f>source!I12/metric!$V$2</f>
@@ -2786,9 +2714,8 @@
         <f>source!A13/metric!$W$2</f>
         <v>59.435999909657284</v>
       </c>
-      <c r="B13">
-        <f>source!B13</f>
-        <v>0</v>
+      <c r="B13" s="14">
+        <v>2.85</v>
       </c>
       <c r="C13">
         <f>source!C13</f>
@@ -2802,9 +2729,8 @@
         <f>source!E13</f>
         <v>3.17</v>
       </c>
-      <c r="F13">
-        <f>source!F13</f>
-        <v>0</v>
+      <c r="F13" s="14">
+        <v>3.65</v>
       </c>
       <c r="I13">
         <f>source!I13/metric!$V$2</f>
@@ -2824,9 +2750,8 @@
         <f>source!A14/metric!$W$2</f>
         <v>64.007999902707851</v>
       </c>
-      <c r="B14">
-        <f>source!B14</f>
-        <v>0</v>
+      <c r="B14" s="14">
+        <v>2.86</v>
       </c>
       <c r="C14">
         <f>source!C14</f>
@@ -2840,9 +2765,8 @@
         <f>source!E14</f>
         <v>3.19</v>
       </c>
-      <c r="F14">
-        <f>source!F14</f>
-        <v>0</v>
+      <c r="F14" s="14">
+        <v>3.7</v>
       </c>
       <c r="I14">
         <f>source!I14/metric!$V$2</f>
@@ -2862,9 +2786,8 @@
         <f>source!A15/metric!$W$2</f>
         <v>68.579999895758405</v>
       </c>
-      <c r="B15">
-        <f>source!B15</f>
-        <v>0</v>
+      <c r="B15" s="14">
+        <v>2.87</v>
       </c>
       <c r="C15">
         <f>source!C15</f>
@@ -2878,9 +2801,8 @@
         <f>source!E15</f>
         <v>3.22</v>
       </c>
-      <c r="F15">
-        <f>source!F15</f>
-        <v>0</v>
+      <c r="F15" s="14">
+        <v>3.7</v>
       </c>
       <c r="I15">
         <f>source!I15/metric!$V$2</f>
@@ -2900,9 +2822,8 @@
         <f>source!A16/metric!$W$2</f>
         <v>73.151999888808973</v>
       </c>
-      <c r="B16">
-        <f>source!B16</f>
-        <v>0</v>
+      <c r="B16" s="14">
+        <v>2.88</v>
       </c>
       <c r="C16">
         <f>source!C16</f>
@@ -2916,9 +2837,8 @@
         <f>source!E16</f>
         <v>3.24</v>
       </c>
-      <c r="F16">
-        <f>source!F16</f>
-        <v>0</v>
+      <c r="F16" s="14">
+        <v>3.7</v>
       </c>
       <c r="I16">
         <f>source!I16/metric!$V$2</f>
@@ -2938,9 +2858,8 @@
         <f>source!A17/metric!$W$2</f>
         <v>77.723999881859527</v>
       </c>
-      <c r="B17">
-        <f>source!B17</f>
-        <v>0</v>
+      <c r="B17" s="14">
+        <v>2.89</v>
       </c>
       <c r="C17">
         <f>source!C17</f>
@@ -2954,9 +2873,8 @@
         <f>source!E17</f>
         <v>3.24</v>
       </c>
-      <c r="F17">
-        <f>source!F17</f>
-        <v>0</v>
+      <c r="F17" s="14">
+        <v>3.75</v>
       </c>
       <c r="I17">
         <f>source!I17/metric!$V$2</f>
@@ -2976,9 +2894,8 @@
         <f>source!A18/metric!$W$2</f>
         <v>82.295999874910095</v>
       </c>
-      <c r="B18">
-        <f>source!B18</f>
-        <v>0</v>
+      <c r="B18" s="14">
+        <v>2.9</v>
       </c>
       <c r="C18">
         <f>source!C18</f>
@@ -2992,9 +2909,8 @@
         <f>source!E18</f>
         <v>3.23</v>
       </c>
-      <c r="F18">
-        <f>source!F18</f>
-        <v>0</v>
+      <c r="F18" s="14">
+        <v>3.75</v>
       </c>
       <c r="M18" s="12">
         <f t="shared" si="0"/>
@@ -3006,9 +2922,8 @@
         <f>source!A19/metric!$W$2</f>
         <v>86.867999867960648</v>
       </c>
-      <c r="B19">
-        <f>source!B19</f>
-        <v>0</v>
+      <c r="B19" s="14">
+        <v>2.91</v>
       </c>
       <c r="C19">
         <f>source!C19</f>
@@ -3022,9 +2937,8 @@
         <f>source!E19</f>
         <v>3.23</v>
       </c>
-      <c r="F19">
-        <f>source!F19</f>
-        <v>0</v>
+      <c r="F19" s="14">
+        <v>3.75</v>
       </c>
       <c r="M19" s="12">
         <f t="shared" si="0"/>
@@ -4418,7 +4332,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2D2087ED-886B-44FE-8790-08DCEB73A4B1}">
-  <dimension ref="A1:H47"/>
+  <dimension ref="A1:H258"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.7109375" bestFit="1" customWidth="1"/>
@@ -4431,1131 +4345,3093 @@
     <col min="8" max="8" width="15" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="18" t="s">
-        <v>16</v>
-      </c>
-      <c r="B1" s="19" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1" s="18" t="s">
-        <v>17</v>
-      </c>
-      <c r="D1" s="19" t="s">
-        <v>15</v>
-      </c>
-      <c r="E1" s="18" t="s">
-        <v>18</v>
-      </c>
-      <c r="F1" s="19" t="s">
-        <v>15</v>
-      </c>
-      <c r="G1" s="18" t="s">
-        <v>19</v>
-      </c>
-      <c r="H1" s="19" t="s">
-        <v>15</v>
-      </c>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" s="15" t="str" cm="1">
+        <f t="array" ref="A1:F1">metric!A1:F1</f>
+        <v>DISTANCE</v>
+      </c>
+      <c r="B1" s="15" t="str">
+        <v>TEE</v>
+      </c>
+      <c r="C1" s="15" t="str">
+        <v>FAIRWAY</v>
+      </c>
+      <c r="D1" s="15" t="str">
+        <v>ROUGH</v>
+      </c>
+      <c r="E1" s="15" t="str">
+        <v>SAND</v>
+      </c>
+      <c r="F1" s="15" t="str">
+        <v>RECOVERY</v>
+      </c>
+      <c r="G1" s="15"/>
+      <c r="H1" s="15"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2" s="14">
-        <f>metric!A20</f>
+      <c r="A2" s="15" cm="1">
+        <f t="array" ref="A2:F2">metric!A2:F2</f>
+        <v>9.1439999861011216</v>
+      </c>
+      <c r="B2" s="15">
+        <v>2.74</v>
+      </c>
+      <c r="C2" s="15">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="D2" s="15">
+        <v>2.4900000000000002</v>
+      </c>
+      <c r="E2" s="15">
+        <v>2.41</v>
+      </c>
+      <c r="F2" s="15">
+        <v>3.5</v>
+      </c>
+      <c r="G2" s="16"/>
+      <c r="H2" s="16"/>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" s="15" cm="1">
+        <f t="array" ref="A3:F3">metric!A3:F3</f>
+        <v>13.715999979151681</v>
+      </c>
+      <c r="B3" s="15">
+        <v>2.75</v>
+      </c>
+      <c r="C3" s="15">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="D3" s="15">
+        <v>2.54</v>
+      </c>
+      <c r="E3" s="15">
+        <v>2.4700000000000002</v>
+      </c>
+      <c r="F3" s="15">
+        <v>3.5</v>
+      </c>
+      <c r="G3" s="16"/>
+      <c r="H3" s="16"/>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" s="15" cm="1">
+        <f t="array" ref="A4:F4">metric!A4:F4</f>
+        <v>18.287999972202243</v>
+      </c>
+      <c r="B4" s="15">
+        <v>2.76</v>
+      </c>
+      <c r="C4" s="15">
+        <v>2.4</v>
+      </c>
+      <c r="D4" s="15">
+        <v>2.59</v>
+      </c>
+      <c r="E4" s="15">
+        <v>2.5299999999999998</v>
+      </c>
+      <c r="F4" s="15">
+        <v>3.5</v>
+      </c>
+      <c r="G4" s="16"/>
+      <c r="H4" s="16"/>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" s="15" cm="1">
+        <f t="array" ref="A5:F5">metric!A5:F5</f>
+        <v>22.859999965252801</v>
+      </c>
+      <c r="B5" s="15">
+        <v>2.77</v>
+      </c>
+      <c r="C5" s="15">
+        <v>2.4500000000000002</v>
+      </c>
+      <c r="D5" s="15">
+        <v>2.64</v>
+      </c>
+      <c r="E5" s="15">
+        <v>2.59</v>
+      </c>
+      <c r="F5" s="15">
+        <v>3.55</v>
+      </c>
+      <c r="G5" s="16"/>
+      <c r="H5" s="16"/>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" s="15" cm="1">
+        <f t="array" ref="A6:F6">metric!A6:F6</f>
+        <v>27.431999958303361</v>
+      </c>
+      <c r="B6" s="15">
+        <v>2.78</v>
+      </c>
+      <c r="C6" s="15">
+        <v>2.5</v>
+      </c>
+      <c r="D6" s="15">
+        <v>2.69</v>
+      </c>
+      <c r="E6" s="15">
+        <v>2.67</v>
+      </c>
+      <c r="F6" s="15">
+        <v>3.55</v>
+      </c>
+      <c r="G6" s="16"/>
+      <c r="H6" s="16"/>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" s="15" cm="1">
+        <f t="array" ref="A7:F7">metric!A7:F7</f>
+        <v>32.003999951353926</v>
+      </c>
+      <c r="B7" s="15">
+        <v>2.79</v>
+      </c>
+      <c r="C7" s="15">
+        <v>2.5499999999999998</v>
+      </c>
+      <c r="D7" s="15">
+        <v>2.74</v>
+      </c>
+      <c r="E7" s="15">
+        <v>2.76</v>
+      </c>
+      <c r="F7" s="15">
+        <v>3.55</v>
+      </c>
+      <c r="G7" s="16"/>
+      <c r="H7" s="16"/>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" s="15" cm="1">
+        <f t="array" ref="A8:F8">metric!A8:F8</f>
+        <v>36.575999944404487</v>
+      </c>
+      <c r="B8" s="15">
+        <v>2.8</v>
+      </c>
+      <c r="C8" s="15">
+        <v>2.6</v>
+      </c>
+      <c r="D8" s="15">
+        <v>2.78</v>
+      </c>
+      <c r="E8" s="15">
+        <v>2.82</v>
+      </c>
+      <c r="F8" s="15">
+        <v>3.6</v>
+      </c>
+      <c r="G8" s="16"/>
+      <c r="H8" s="16"/>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" s="15" cm="1">
+        <f t="array" ref="A9:F9">metric!A9:F9</f>
+        <v>41.147999937455047</v>
+      </c>
+      <c r="B9" s="15">
+        <v>2.81</v>
+      </c>
+      <c r="C9" s="15">
+        <v>2.62</v>
+      </c>
+      <c r="D9" s="15">
+        <v>2.82</v>
+      </c>
+      <c r="E9" s="15">
+        <v>2.9</v>
+      </c>
+      <c r="F9" s="15">
+        <v>3.6</v>
+      </c>
+      <c r="G9" s="16"/>
+      <c r="H9" s="16"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" s="15" cm="1">
+        <f t="array" ref="A10:F10">metric!A10:F10</f>
+        <v>45.719999930505601</v>
+      </c>
+      <c r="B10" s="15">
+        <v>2.82</v>
+      </c>
+      <c r="C10" s="15">
+        <v>2.65</v>
+      </c>
+      <c r="D10" s="15">
+        <v>2.85</v>
+      </c>
+      <c r="E10" s="15">
+        <v>2.98</v>
+      </c>
+      <c r="F10" s="15">
+        <v>3.6</v>
+      </c>
+      <c r="G10" s="16"/>
+      <c r="H10" s="16"/>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" s="15" cm="1">
+        <f t="array" ref="A11:F11">metric!A11:F11</f>
+        <v>50.291999923556162</v>
+      </c>
+      <c r="B11" s="15">
+        <v>2.83</v>
+      </c>
+      <c r="C11" s="15">
+        <v>2.67</v>
+      </c>
+      <c r="D11" s="15">
+        <v>2.88</v>
+      </c>
+      <c r="E11" s="15">
+        <v>3.07</v>
+      </c>
+      <c r="F11" s="15">
+        <v>3.65</v>
+      </c>
+      <c r="G11" s="16"/>
+      <c r="H11" s="16"/>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" s="15" cm="1">
+        <f t="array" ref="A12:F12">metric!A12:F12</f>
+        <v>54.863999916606723</v>
+      </c>
+      <c r="B12" s="15">
+        <v>2.84</v>
+      </c>
+      <c r="C12" s="15">
+        <v>2.7</v>
+      </c>
+      <c r="D12" s="15">
+        <v>2.91</v>
+      </c>
+      <c r="E12" s="15">
+        <v>3.15</v>
+      </c>
+      <c r="F12" s="15">
+        <v>3.65</v>
+      </c>
+      <c r="G12" s="16"/>
+      <c r="H12" s="16"/>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" s="15" cm="1">
+        <f t="array" ref="A13:F13">metric!A13:F13</f>
+        <v>59.435999909657284</v>
+      </c>
+      <c r="B13" s="15">
+        <v>2.85</v>
+      </c>
+      <c r="C13" s="15">
+        <v>2.72</v>
+      </c>
+      <c r="D13" s="15">
+        <v>2.92</v>
+      </c>
+      <c r="E13" s="15">
+        <v>3.17</v>
+      </c>
+      <c r="F13" s="15">
+        <v>3.65</v>
+      </c>
+      <c r="G13" s="16"/>
+      <c r="H13" s="16"/>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" s="15" cm="1">
+        <f t="array" ref="A14:F14">metric!A14:F14</f>
+        <v>64.007999902707851</v>
+      </c>
+      <c r="B14" s="15">
+        <v>2.86</v>
+      </c>
+      <c r="C14" s="15">
+        <v>2.73</v>
+      </c>
+      <c r="D14" s="15">
+        <v>2.93</v>
+      </c>
+      <c r="E14" s="15">
+        <v>3.19</v>
+      </c>
+      <c r="F14" s="15">
+        <v>3.7</v>
+      </c>
+      <c r="G14" s="16"/>
+      <c r="H14" s="16"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" s="15" cm="1">
+        <f t="array" ref="A15:F15">metric!A15:F15</f>
+        <v>68.579999895758405</v>
+      </c>
+      <c r="B15" s="15">
+        <v>2.87</v>
+      </c>
+      <c r="C15" s="15">
+        <v>2.74</v>
+      </c>
+      <c r="D15" s="15">
+        <v>2.95</v>
+      </c>
+      <c r="E15" s="15">
+        <v>3.22</v>
+      </c>
+      <c r="F15" s="15">
+        <v>3.7</v>
+      </c>
+      <c r="G15" s="16"/>
+      <c r="H15" s="16"/>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" s="15" cm="1">
+        <f t="array" ref="A16:F16">metric!A16:F16</f>
+        <v>73.151999888808973</v>
+      </c>
+      <c r="B16" s="15">
+        <v>2.88</v>
+      </c>
+      <c r="C16" s="15">
+        <v>2.75</v>
+      </c>
+      <c r="D16" s="15">
+        <v>2.96</v>
+      </c>
+      <c r="E16" s="15">
+        <v>3.24</v>
+      </c>
+      <c r="F16" s="15">
+        <v>3.7</v>
+      </c>
+      <c r="G16" s="16"/>
+      <c r="H16" s="16"/>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" s="15" cm="1">
+        <f t="array" ref="A17:F17">metric!A17:F17</f>
+        <v>77.723999881859527</v>
+      </c>
+      <c r="B17" s="15">
+        <v>2.89</v>
+      </c>
+      <c r="C17" s="15">
+        <v>2.77</v>
+      </c>
+      <c r="D17" s="15">
+        <v>2.97</v>
+      </c>
+      <c r="E17" s="15">
+        <v>3.24</v>
+      </c>
+      <c r="F17" s="15">
+        <v>3.75</v>
+      </c>
+      <c r="G17" s="16"/>
+      <c r="H17" s="16"/>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" s="15" cm="1">
+        <f t="array" ref="A18:F18">metric!A18:F18</f>
+        <v>82.295999874910095</v>
+      </c>
+      <c r="B18" s="15">
+        <v>2.9</v>
+      </c>
+      <c r="C18" s="15">
+        <v>2.78</v>
+      </c>
+      <c r="D18" s="15">
+        <v>2.99</v>
+      </c>
+      <c r="E18" s="15">
+        <v>3.23</v>
+      </c>
+      <c r="F18" s="15">
+        <v>3.75</v>
+      </c>
+      <c r="G18" s="16"/>
+      <c r="H18" s="16"/>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" s="15" cm="1">
+        <f t="array" ref="A19:F19">metric!A19:F19</f>
+        <v>86.867999867960648</v>
+      </c>
+      <c r="B19" s="15">
+        <v>2.91</v>
+      </c>
+      <c r="C19" s="15">
+        <v>2.79</v>
+      </c>
+      <c r="D19" s="15">
+        <v>3.01</v>
+      </c>
+      <c r="E19" s="15">
+        <v>3.23</v>
+      </c>
+      <c r="F19" s="15">
+        <v>3.75</v>
+      </c>
+      <c r="G19" s="16"/>
+      <c r="H19" s="16"/>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" s="15" cm="1">
+        <f t="array" ref="A20:F20">metric!A20:F20</f>
         <v>91.439999861011202</v>
       </c>
-      <c r="B2" s="15">
-        <f>metric!B20</f>
+      <c r="B20" s="15">
         <v>2.92</v>
       </c>
-      <c r="C2" s="14">
-        <f>metric!A20</f>
-        <v>91.439999861011202</v>
-      </c>
-      <c r="D2" s="15">
-        <f>metric!L20</f>
-        <v>3.0166666666666671</v>
-      </c>
-      <c r="E2" s="14">
-        <f>metric!A2</f>
-        <v>9.1439999861011216</v>
-      </c>
-      <c r="F2" s="15">
-        <f>metric!M2</f>
-        <v>2.3666666666666667</v>
-      </c>
-      <c r="G2" s="14">
-        <f>metric!I2</f>
+      <c r="C20" s="15">
+        <v>2.8</v>
+      </c>
+      <c r="D20" s="15">
+        <v>3.02</v>
+      </c>
+      <c r="E20" s="15">
+        <v>3.23</v>
+      </c>
+      <c r="F20" s="15">
+        <v>3.8</v>
+      </c>
+      <c r="G20" s="16"/>
+      <c r="H20" s="16"/>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21" s="15" cm="1">
+        <f t="array" ref="A21:F21">metric!A21:F21</f>
+        <v>96.01199985406177</v>
+      </c>
+      <c r="B21" s="15">
+        <v>2.93</v>
+      </c>
+      <c r="C21" s="15">
+        <v>2.81</v>
+      </c>
+      <c r="D21" s="15">
+        <v>3.03</v>
+      </c>
+      <c r="E21" s="15">
+        <v>3.23</v>
+      </c>
+      <c r="F21" s="15">
+        <v>3.8</v>
+      </c>
+      <c r="G21" s="16"/>
+      <c r="H21" s="16"/>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A22" s="15" cm="1">
+        <f t="array" ref="A22:F22">metric!A22:F22</f>
+        <v>100.58399984711232</v>
+      </c>
+      <c r="B22" s="15">
+        <v>2.95</v>
+      </c>
+      <c r="C22" s="15">
+        <v>2.83</v>
+      </c>
+      <c r="D22" s="15">
+        <v>3.04</v>
+      </c>
+      <c r="E22" s="15">
+        <v>3.22</v>
+      </c>
+      <c r="F22" s="15">
+        <v>3.8</v>
+      </c>
+      <c r="G22" s="16"/>
+      <c r="H22" s="16"/>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23" s="15" cm="1">
+        <f t="array" ref="A23:F23">metric!A23:F23</f>
+        <v>105.15599984016289</v>
+      </c>
+      <c r="B23" s="15">
+        <v>2.97</v>
+      </c>
+      <c r="C23" s="15">
+        <v>2.84</v>
+      </c>
+      <c r="D23" s="15">
+        <v>3.06</v>
+      </c>
+      <c r="E23" s="15">
+        <v>3.21</v>
+      </c>
+      <c r="F23" s="15">
+        <v>3.8</v>
+      </c>
+      <c r="G23" s="16"/>
+      <c r="H23" s="16"/>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24" s="15" cm="1">
+        <f t="array" ref="A24:F24">metric!A24:F24</f>
+        <v>109.72799983321345</v>
+      </c>
+      <c r="B24" s="15">
+        <v>2.99</v>
+      </c>
+      <c r="C24" s="15">
+        <v>2.85</v>
+      </c>
+      <c r="D24" s="15">
+        <v>3.08</v>
+      </c>
+      <c r="E24" s="15">
+        <v>3.21</v>
+      </c>
+      <c r="F24" s="15">
+        <v>3.78</v>
+      </c>
+      <c r="G24" s="16"/>
+      <c r="H24" s="16"/>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A25" s="15" cm="1">
+        <f t="array" ref="A25:F25">metric!A25:F25</f>
+        <v>114.29999982626401</v>
+      </c>
+      <c r="B25" s="15">
+        <v>2.99</v>
+      </c>
+      <c r="C25" s="15">
+        <v>2.86</v>
+      </c>
+      <c r="D25" s="15">
+        <v>3.09</v>
+      </c>
+      <c r="E25" s="15">
+        <v>3.21</v>
+      </c>
+      <c r="F25" s="15">
+        <v>3.78</v>
+      </c>
+      <c r="G25" s="16"/>
+      <c r="H25" s="16"/>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A26" s="15" cm="1">
+        <f t="array" ref="A26:F26">metric!A26:F26</f>
+        <v>118.87199981931457</v>
+      </c>
+      <c r="B26" s="15">
+        <v>2.97</v>
+      </c>
+      <c r="C26" s="15">
+        <v>2.88</v>
+      </c>
+      <c r="D26" s="15">
+        <v>3.11</v>
+      </c>
+      <c r="E26" s="15">
+        <v>3.21</v>
+      </c>
+      <c r="F26" s="15">
+        <v>3.78</v>
+      </c>
+      <c r="G26" s="16"/>
+      <c r="H26" s="16"/>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A27" s="15" cm="1">
+        <f t="array" ref="A27:F27">metric!A27:F27</f>
+        <v>123.44399981236513</v>
+      </c>
+      <c r="B27" s="15">
+        <v>2.97</v>
+      </c>
+      <c r="C27" s="15">
+        <v>2.9</v>
+      </c>
+      <c r="D27" s="15">
+        <v>3.13</v>
+      </c>
+      <c r="E27" s="15">
+        <v>3.22</v>
+      </c>
+      <c r="F27" s="15">
+        <v>3.78</v>
+      </c>
+      <c r="G27" s="16"/>
+      <c r="H27" s="16"/>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A28" s="15" cm="1">
+        <f t="array" ref="A28:F28">metric!A28:F28</f>
+        <v>128.0159998054157</v>
+      </c>
+      <c r="B28" s="15">
+        <v>2.97</v>
+      </c>
+      <c r="C28" s="15">
+        <v>2.91</v>
+      </c>
+      <c r="D28" s="15">
+        <v>3.15</v>
+      </c>
+      <c r="E28" s="15">
+        <v>3.22</v>
+      </c>
+      <c r="F28" s="15">
+        <v>3.8</v>
+      </c>
+      <c r="G28" s="16"/>
+      <c r="H28" s="16"/>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A29" s="15" cm="1">
+        <f t="array" ref="A29:F29">metric!A29:F29</f>
+        <v>132.58799979846626</v>
+      </c>
+      <c r="B29" s="15">
+        <v>2.97</v>
+      </c>
+      <c r="C29" s="15">
+        <v>2.93</v>
+      </c>
+      <c r="D29" s="15">
+        <v>3.17</v>
+      </c>
+      <c r="E29" s="15">
+        <v>3.23</v>
+      </c>
+      <c r="F29" s="15">
+        <v>3.8</v>
+      </c>
+      <c r="G29" s="16"/>
+      <c r="H29" s="16"/>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A30" s="15" cm="1">
+        <f t="array" ref="A30:F30">metric!A30:F30</f>
+        <v>137.15999979151681</v>
+      </c>
+      <c r="B30" s="15">
+        <v>2.99</v>
+      </c>
+      <c r="C30" s="15">
+        <v>2.95</v>
+      </c>
+      <c r="D30" s="15">
+        <v>3.19</v>
+      </c>
+      <c r="E30" s="15">
+        <v>3.25</v>
+      </c>
+      <c r="F30" s="15">
+        <v>3.8</v>
+      </c>
+      <c r="G30" s="16"/>
+      <c r="H30" s="16"/>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A31" s="15" cm="1">
+        <f t="array" ref="A31:F31">metric!A31:F31</f>
+        <v>141.73199978456736</v>
+      </c>
+      <c r="B31" s="15">
+        <v>2.99</v>
+      </c>
+      <c r="C31" s="15">
+        <v>2.97</v>
+      </c>
+      <c r="D31" s="15">
+        <v>3.21</v>
+      </c>
+      <c r="E31" s="15">
+        <v>3.26</v>
+      </c>
+      <c r="F31" s="15">
+        <v>3.8</v>
+      </c>
+      <c r="G31" s="16"/>
+      <c r="H31" s="16"/>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A32" s="15" cm="1">
+        <f t="array" ref="A32:F32">metric!A32:F32</f>
+        <v>146.30399977761795</v>
+      </c>
+      <c r="B32" s="15">
+        <v>2.99</v>
+      </c>
+      <c r="C32" s="15">
+        <v>2.98</v>
+      </c>
+      <c r="D32" s="15">
+        <v>3.23</v>
+      </c>
+      <c r="E32" s="15">
+        <v>3.28</v>
+      </c>
+      <c r="F32" s="15">
+        <v>3.81</v>
+      </c>
+      <c r="G32" s="16"/>
+      <c r="H32" s="16"/>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A33" s="15" cm="1">
+        <f t="array" ref="A33:F33">metric!A33:F33</f>
+        <v>150.8759997706685</v>
+      </c>
+      <c r="B33" s="15">
+        <v>3.01</v>
+      </c>
+      <c r="C33" s="15">
+        <v>3</v>
+      </c>
+      <c r="D33" s="15">
+        <v>3.25</v>
+      </c>
+      <c r="E33" s="15">
+        <v>3.3</v>
+      </c>
+      <c r="F33" s="15">
+        <v>3.81</v>
+      </c>
+      <c r="G33" s="16"/>
+      <c r="H33" s="16"/>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A34" s="15" cm="1">
+        <f t="array" ref="A34:F34">metric!A34:F34</f>
+        <v>155.44799976371905</v>
+      </c>
+      <c r="B34" s="15">
+        <v>3.02</v>
+      </c>
+      <c r="C34" s="15">
+        <v>3.03</v>
+      </c>
+      <c r="D34" s="15">
+        <v>3.27</v>
+      </c>
+      <c r="E34" s="15">
+        <v>3.33</v>
+      </c>
+      <c r="F34" s="15">
+        <v>3.81</v>
+      </c>
+      <c r="G34" s="16"/>
+      <c r="H34" s="16"/>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A35" s="15" cm="1">
+        <f t="array" ref="A35:F35">metric!A35:F35</f>
+        <v>160.01999975676961</v>
+      </c>
+      <c r="B35" s="15">
+        <v>3.04</v>
+      </c>
+      <c r="C35" s="15">
+        <v>3.06</v>
+      </c>
+      <c r="D35" s="15">
+        <v>3.29</v>
+      </c>
+      <c r="E35" s="15">
+        <v>3.36</v>
+      </c>
+      <c r="F35" s="15">
+        <v>3.81</v>
+      </c>
+      <c r="G35" s="16"/>
+      <c r="H35" s="16"/>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A36" s="15" cm="1">
+        <f t="array" ref="A36:F36">metric!A36:F36</f>
+        <v>164.59199974982019</v>
+      </c>
+      <c r="B36" s="15">
+        <v>3.05</v>
+      </c>
+      <c r="C36" s="15">
+        <v>3.08</v>
+      </c>
+      <c r="D36" s="15">
+        <v>3.31</v>
+      </c>
+      <c r="E36" s="15">
+        <v>3.4</v>
+      </c>
+      <c r="F36" s="15">
+        <v>3.82</v>
+      </c>
+      <c r="G36" s="16"/>
+      <c r="H36" s="16"/>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A37" s="15" cm="1">
+        <f t="array" ref="A37:F37">metric!A37:F37</f>
+        <v>169.16399974287074</v>
+      </c>
+      <c r="B37" s="15">
+        <v>3.07</v>
+      </c>
+      <c r="C37" s="15">
+        <v>3.11</v>
+      </c>
+      <c r="D37" s="15">
+        <v>3.34</v>
+      </c>
+      <c r="E37" s="15">
+        <v>3.43</v>
+      </c>
+      <c r="F37" s="15">
+        <v>3.83</v>
+      </c>
+      <c r="G37" s="16"/>
+      <c r="H37" s="16"/>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A38" s="15" cm="1">
+        <f t="array" ref="A38:F38">metric!A38:F38</f>
+        <v>173.7359997359213</v>
+      </c>
+      <c r="B38" s="15">
+        <v>3.09</v>
+      </c>
+      <c r="C38" s="15">
+        <v>3.13</v>
+      </c>
+      <c r="D38" s="15">
+        <v>3.37</v>
+      </c>
+      <c r="E38" s="15">
+        <v>3.47</v>
+      </c>
+      <c r="F38" s="15">
+        <v>3.84</v>
+      </c>
+      <c r="G38" s="16"/>
+      <c r="H38" s="16"/>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A39" s="15" cm="1">
+        <f t="array" ref="A39:F39">metric!A39:F39</f>
+        <v>178.30799972897185</v>
+      </c>
+      <c r="B39" s="15">
+        <v>3.11</v>
+      </c>
+      <c r="C39" s="15">
+        <v>3.16</v>
+      </c>
+      <c r="D39" s="15">
+        <v>3.4</v>
+      </c>
+      <c r="E39" s="15">
+        <v>3.51</v>
+      </c>
+      <c r="F39" s="15">
+        <v>3.86</v>
+      </c>
+      <c r="G39" s="16"/>
+      <c r="H39" s="16"/>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A40" s="15" cm="1">
+        <f t="array" ref="A40:F40">metric!A40:F40</f>
+        <v>182.8799997220224</v>
+      </c>
+      <c r="B40" s="15">
+        <v>3.12</v>
+      </c>
+      <c r="C40" s="15">
+        <v>3.19</v>
+      </c>
+      <c r="D40" s="15">
+        <v>3.42</v>
+      </c>
+      <c r="E40" s="15">
+        <v>3.55</v>
+      </c>
+      <c r="F40" s="15">
+        <v>3.87</v>
+      </c>
+      <c r="G40" s="16"/>
+      <c r="H40" s="16"/>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A41" s="15" cm="1">
+        <f t="array" ref="A41:F41">metric!A41:F41</f>
+        <v>192.02399970812354</v>
+      </c>
+      <c r="B41" s="15">
+        <v>3.14</v>
+      </c>
+      <c r="C41" s="15">
+        <v>3.26</v>
+      </c>
+      <c r="D41" s="15">
+        <v>3.48</v>
+      </c>
+      <c r="E41" s="15">
+        <v>3.62</v>
+      </c>
+      <c r="F41" s="15">
+        <v>3.89</v>
+      </c>
+      <c r="G41" s="16"/>
+      <c r="H41" s="16"/>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A42" s="15" cm="1">
+        <f t="array" ref="A42:F42">metric!A42:F42</f>
+        <v>201.16799969422465</v>
+      </c>
+      <c r="B42" s="15">
+        <v>3.17</v>
+      </c>
+      <c r="C42" s="15">
+        <v>3.32</v>
+      </c>
+      <c r="D42" s="15">
+        <v>3.53</v>
+      </c>
+      <c r="E42" s="15">
+        <v>3.7</v>
+      </c>
+      <c r="F42" s="15">
+        <v>3.92</v>
+      </c>
+      <c r="G42" s="16"/>
+      <c r="H42" s="16"/>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A43" s="15" cm="1">
+        <f t="array" ref="A43:F43">metric!A43:F43</f>
+        <v>210.31199968032578</v>
+      </c>
+      <c r="B43" s="15">
+        <v>3.21</v>
+      </c>
+      <c r="C43" s="15">
+        <v>3.39</v>
+      </c>
+      <c r="D43" s="15">
+        <v>3.8</v>
+      </c>
+      <c r="E43" s="15">
+        <v>3.77</v>
+      </c>
+      <c r="F43" s="15">
+        <v>3.95</v>
+      </c>
+      <c r="G43" s="16"/>
+      <c r="H43" s="16"/>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A44" s="15" cm="1">
+        <f t="array" ref="A44:F44">metric!A44:F44</f>
+        <v>219.45599966642689</v>
+      </c>
+      <c r="B44" s="15">
+        <v>3.25</v>
+      </c>
+      <c r="C44" s="15">
+        <v>3.45</v>
+      </c>
+      <c r="D44" s="15">
+        <v>3.64</v>
+      </c>
+      <c r="E44" s="15">
+        <v>3.84</v>
+      </c>
+      <c r="F44" s="15">
+        <v>3.97</v>
+      </c>
+      <c r="G44" s="16"/>
+      <c r="H44" s="16"/>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A45" s="15" cm="1">
+        <f t="array" ref="A45:F45">metric!A45:F45</f>
+        <v>228.59999965252803</v>
+      </c>
+      <c r="B45" s="15">
+        <v>3.35</v>
+      </c>
+      <c r="C45" s="15">
+        <v>3.52</v>
+      </c>
+      <c r="D45" s="15">
+        <v>3.69</v>
+      </c>
+      <c r="E45" s="15">
+        <v>3.88</v>
+      </c>
+      <c r="F45" s="15">
+        <v>4</v>
+      </c>
+      <c r="G45" s="16"/>
+      <c r="H45" s="16"/>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A46" s="15" cm="1">
+        <f t="array" ref="A46:F46">metric!A46:F46</f>
+        <v>237.74399963862913</v>
+      </c>
+      <c r="B46" s="15">
+        <v>3.45</v>
+      </c>
+      <c r="C46" s="15">
+        <v>3.58</v>
+      </c>
+      <c r="D46" s="15">
+        <v>3.74</v>
+      </c>
+      <c r="E46" s="15">
+        <v>3.93</v>
+      </c>
+      <c r="F46" s="15">
+        <v>4.03</v>
+      </c>
+      <c r="G46" s="16"/>
+      <c r="H46" s="16"/>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A47" s="15" cm="1">
+        <f t="array" ref="A47:F47">metric!A47:F47</f>
+        <v>246.88799962473027</v>
+      </c>
+      <c r="B47" s="15">
+        <v>3.55</v>
+      </c>
+      <c r="C47" s="15">
+        <v>3.63</v>
+      </c>
+      <c r="D47" s="15">
+        <v>3.78</v>
+      </c>
+      <c r="E47" s="15">
+        <v>3.96</v>
+      </c>
+      <c r="F47" s="15">
+        <v>4.07</v>
+      </c>
+      <c r="G47" s="16"/>
+      <c r="H47" s="16"/>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A48" s="15" cm="1">
+        <f t="array" ref="A48:F48">metric!A48:F48</f>
+        <v>256.03199961083141</v>
+      </c>
+      <c r="B48" s="15">
+        <v>3.65</v>
+      </c>
+      <c r="C48" s="15">
+        <v>3.69</v>
+      </c>
+      <c r="D48" s="15">
+        <v>3.83</v>
+      </c>
+      <c r="E48" s="15">
+        <v>4</v>
+      </c>
+      <c r="F48" s="15">
+        <v>4.0999999999999996</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" s="15" cm="1">
+        <f t="array" ref="A49:F49">metric!A49:F49</f>
+        <v>265.17599959693251</v>
+      </c>
+      <c r="B49" s="15">
+        <v>3.68</v>
+      </c>
+      <c r="C49" s="15">
+        <v>3.74</v>
+      </c>
+      <c r="D49" s="15">
+        <v>3.87</v>
+      </c>
+      <c r="E49" s="15">
+        <v>4.0199999999999996</v>
+      </c>
+      <c r="F49" s="15">
+        <v>4.1500000000000004</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" s="15" cm="1">
+        <f t="array" ref="A50:F50">metric!A50:F50</f>
+        <v>274.31999958303362</v>
+      </c>
+      <c r="B50" s="15">
+        <v>3.71</v>
+      </c>
+      <c r="C50" s="15">
+        <v>3.78</v>
+      </c>
+      <c r="D50" s="15">
+        <v>3.9</v>
+      </c>
+      <c r="E50" s="15">
+        <v>4.04</v>
+      </c>
+      <c r="F50" s="15">
+        <v>4.2</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" s="15" cm="1">
+        <f t="array" ref="A51:F51">metric!A51:F51</f>
+        <v>292.60799955523589</v>
+      </c>
+      <c r="B51" s="15">
+        <v>3.79</v>
+      </c>
+      <c r="C51" s="15">
+        <v>3.84</v>
+      </c>
+      <c r="D51" s="15">
+        <v>3.95</v>
+      </c>
+      <c r="E51" s="15">
+        <v>4.12</v>
+      </c>
+      <c r="F51" s="15">
+        <v>4.3099999999999996</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" s="15" cm="1">
+        <f t="array" ref="A52:F52">metric!A52:F52</f>
+        <v>310.89599952743811</v>
+      </c>
+      <c r="B52" s="15">
+        <v>3.86</v>
+      </c>
+      <c r="C52" s="15">
+        <v>3.88</v>
+      </c>
+      <c r="D52" s="15">
+        <v>4.0199999999999996</v>
+      </c>
+      <c r="E52" s="15">
+        <v>4.26</v>
+      </c>
+      <c r="F52" s="15">
+        <v>4.4400000000000004</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" s="15" cm="1">
+        <f t="array" ref="A53:F53">metric!A53:F53</f>
+        <v>329.18399949964038</v>
+      </c>
+      <c r="B53" s="15">
+        <v>3.92</v>
+      </c>
+      <c r="C53" s="15">
+        <v>3.95</v>
+      </c>
+      <c r="D53" s="15">
+        <v>4.1100000000000003</v>
+      </c>
+      <c r="E53" s="15">
+        <v>4.41</v>
+      </c>
+      <c r="F53" s="15">
+        <v>4.5599999999999996</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" s="15" cm="1">
+        <f t="array" ref="A54:F54">metric!A54:F54</f>
+        <v>347.47199947184259</v>
+      </c>
+      <c r="B54" s="15">
+        <v>3.96</v>
+      </c>
+      <c r="C54" s="15">
+        <v>4.03</v>
+      </c>
+      <c r="D54" s="15">
+        <v>4.21</v>
+      </c>
+      <c r="E54" s="15">
+        <v>4.55</v>
+      </c>
+      <c r="F54" s="15">
+        <v>4.66</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" s="15" cm="1">
+        <f t="array" ref="A55:F55">metric!A55:F55</f>
+        <v>365.75999944404481</v>
+      </c>
+      <c r="B55" s="15">
+        <v>3.99</v>
+      </c>
+      <c r="C55" s="15">
+        <v>4.1100000000000003</v>
+      </c>
+      <c r="D55" s="15">
+        <v>4.3</v>
+      </c>
+      <c r="E55" s="15">
+        <v>4.6900000000000004</v>
+      </c>
+      <c r="F55" s="15">
+        <v>4.75</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" s="15" cm="1">
+        <f t="array" ref="A56:F56">metric!A56:F56</f>
+        <v>384.04799941624708</v>
+      </c>
+      <c r="B56" s="15">
+        <v>4.0199999999999996</v>
+      </c>
+      <c r="C56" s="15">
+        <v>4.1500000000000004</v>
+      </c>
+      <c r="D56" s="15">
+        <v>4.34</v>
+      </c>
+      <c r="E56" s="15">
+        <v>4.7300000000000004</v>
+      </c>
+      <c r="F56" s="15">
+        <v>4.79</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" s="15" cm="1">
+        <f t="array" ref="A57:F57">metric!A57:F57</f>
+        <v>402.3359993884493</v>
+      </c>
+      <c r="B57" s="15">
+        <v>4.08</v>
+      </c>
+      <c r="C57" s="15">
+        <v>4.2</v>
+      </c>
+      <c r="D57" s="15">
+        <v>4.3899999999999997</v>
+      </c>
+      <c r="E57" s="15">
+        <v>4.78</v>
+      </c>
+      <c r="F57" s="15">
+        <v>4.84</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" s="15" cm="1">
+        <f t="array" ref="A58:F58">metric!A58:F58</f>
+        <v>420.62399936065157</v>
+      </c>
+      <c r="B58" s="15">
+        <v>4.17</v>
+      </c>
+      <c r="C58" s="15">
+        <v>4.29</v>
+      </c>
+      <c r="D58" s="15">
+        <v>4.4800000000000004</v>
+      </c>
+      <c r="E58" s="15">
+        <v>4.87</v>
+      </c>
+      <c r="F58" s="15">
+        <v>4.93</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" s="15" cm="1">
+        <f t="array" ref="A59:F59">metric!A59:F59</f>
+        <v>438.91199933285378</v>
+      </c>
+      <c r="B59" s="15">
+        <v>4.28</v>
+      </c>
+      <c r="C59" s="15">
+        <v>4.4000000000000004</v>
+      </c>
+      <c r="D59" s="15">
+        <v>4.59</v>
+      </c>
+      <c r="E59" s="15">
+        <v>4.9800000000000004</v>
+      </c>
+      <c r="F59" s="15">
+        <v>5.04</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" s="15" cm="1">
+        <f t="array" ref="A60:F60">metric!A60:F60</f>
+        <v>457.19999930505605</v>
+      </c>
+      <c r="B60" s="15">
+        <v>4.41</v>
+      </c>
+      <c r="C60" s="15">
+        <v>4.53</v>
+      </c>
+      <c r="D60" s="15">
+        <v>4.72</v>
+      </c>
+      <c r="E60" s="15">
+        <v>5.1100000000000003</v>
+      </c>
+      <c r="F60" s="15">
+        <v>5.17</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" s="15" cm="1">
+        <f t="array" ref="A61:F61">metric!A61:F61</f>
+        <v>475.48799927725827</v>
+      </c>
+      <c r="B61" s="15">
+        <v>4.54</v>
+      </c>
+      <c r="C61" s="15">
+        <v>4.8499999999999996</v>
+      </c>
+      <c r="D61" s="15">
+        <v>4.8499999999999996</v>
+      </c>
+      <c r="E61" s="15">
+        <v>5.24</v>
+      </c>
+      <c r="F61" s="15">
+        <v>5.3</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" s="15" cm="1">
+        <f t="array" ref="A62:F62">metric!A62:F62</f>
+        <v>493.77599924946054</v>
+      </c>
+      <c r="B62" s="15">
+        <v>4.6500000000000004</v>
+      </c>
+      <c r="C62" s="15">
+        <v>4.97</v>
+      </c>
+      <c r="D62" s="15">
+        <v>4.97</v>
+      </c>
+      <c r="E62" s="15">
+        <v>5.36</v>
+      </c>
+      <c r="F62" s="15">
+        <v>5.42</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" s="15" cm="1">
+        <f t="array" ref="A63:F63">metric!A63:F63</f>
+        <v>512.06399922166281</v>
+      </c>
+      <c r="B63" s="15">
+        <v>4.74</v>
+      </c>
+      <c r="C63" s="15">
+        <v>5.05</v>
+      </c>
+      <c r="D63" s="15">
+        <v>5.05</v>
+      </c>
+      <c r="E63" s="15">
+        <v>5.44</v>
+      </c>
+      <c r="F63" s="15">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" s="15" cm="1">
+        <f t="array" ref="A64:F64">metric!A64:F64</f>
+        <v>530.35199919386503</v>
+      </c>
+      <c r="B64" s="15">
+        <v>4.79</v>
+      </c>
+      <c r="C64" s="15">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="D64" s="15">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="E64" s="15">
+        <v>5.49</v>
+      </c>
+      <c r="F64" s="15">
+        <v>5.55</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" s="15" cm="1">
+        <f t="array" ref="A65:F65">metric!A65:F65</f>
+        <v>548.63999916606724</v>
+      </c>
+      <c r="B65" s="15">
+        <v>4.82</v>
+      </c>
+      <c r="C65" s="15">
+        <v>5.13</v>
+      </c>
+      <c r="D65" s="15">
+        <v>5.13</v>
+      </c>
+      <c r="E65" s="15">
+        <v>5.52</v>
+      </c>
+      <c r="F65" s="15">
+        <v>5.58</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" s="15"/>
+      <c r="B66" s="15"/>
+      <c r="C66" s="15"/>
+      <c r="D66" s="15"/>
+      <c r="E66" s="15"/>
+      <c r="F66" s="15"/>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A67" s="15" t="str" cm="1">
+        <f t="array" ref="A67:B67">metric!I1:J1</f>
+        <v>DISTANCE</v>
+      </c>
+      <c r="B67" s="15" t="str">
+        <v>GREEN</v>
+      </c>
+      <c r="C67" s="15"/>
+      <c r="D67" s="15"/>
+      <c r="E67" s="15"/>
+      <c r="F67" s="15"/>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A68" s="15" cm="1">
+        <f t="array" ref="A68:B68">metric!I2:J2</f>
         <v>0.304799999536704</v>
       </c>
-      <c r="H2" s="15">
-        <f>metric!J2</f>
+      <c r="B68" s="15">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A3" s="14">
-        <f>metric!A21</f>
-        <v>96.01199985406177</v>
-      </c>
-      <c r="B3" s="15">
-        <f>metric!B21</f>
-        <v>2.93</v>
-      </c>
-      <c r="C3" s="14">
-        <f>metric!A21</f>
-        <v>96.01199985406177</v>
-      </c>
-      <c r="D3" s="15">
-        <f>metric!L21</f>
-        <v>3.0233333333333334</v>
-      </c>
-      <c r="E3" s="14">
-        <f>metric!A3</f>
-        <v>13.715999979151681</v>
-      </c>
-      <c r="F3" s="15">
-        <f>metric!M3</f>
-        <v>2.436666666666667</v>
-      </c>
-      <c r="G3" s="14">
-        <f>metric!I3</f>
+      <c r="C68" s="15"/>
+      <c r="D68" s="15"/>
+      <c r="E68" s="15"/>
+      <c r="F68" s="15"/>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A69" s="15" cm="1">
+        <f t="array" ref="A69:B69">metric!I3:J3</f>
         <v>0.91439999861011201</v>
       </c>
-      <c r="H3" s="15">
-        <f>metric!J3</f>
+      <c r="B69" s="15">
         <v>1.04</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" s="14">
-        <f>metric!A22</f>
-        <v>100.58399984711232</v>
-      </c>
-      <c r="B4" s="15">
-        <f>metric!B22</f>
-        <v>2.95</v>
-      </c>
-      <c r="C4" s="14">
-        <f>metric!A22</f>
-        <v>100.58399984711232</v>
-      </c>
-      <c r="D4" s="15">
-        <f>metric!L22</f>
-        <v>3.03</v>
-      </c>
-      <c r="E4" s="14">
-        <f>metric!A4</f>
-        <v>18.287999972202243</v>
-      </c>
-      <c r="F4" s="15">
-        <f>metric!M4</f>
-        <v>2.5066666666666664</v>
-      </c>
-      <c r="G4" s="14">
-        <f>metric!I4</f>
+      <c r="C69" s="15"/>
+      <c r="D69" s="15"/>
+      <c r="E69" s="15"/>
+      <c r="F69" s="15"/>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A70" s="15" cm="1">
+        <f t="array" ref="A70:B70">metric!I4:J4</f>
         <v>1.219199998146816</v>
       </c>
-      <c r="H4" s="15">
-        <f>metric!J4</f>
+      <c r="B70" s="15">
         <v>1.1299999999999999</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" s="14">
-        <f>metric!A23</f>
-        <v>105.15599984016289</v>
-      </c>
-      <c r="B5" s="15">
-        <f>metric!B23</f>
-        <v>2.97</v>
-      </c>
-      <c r="C5" s="14">
-        <f>metric!A23</f>
-        <v>105.15599984016289</v>
-      </c>
-      <c r="D5" s="15">
-        <f>metric!L23</f>
-        <v>3.0366666666666666</v>
-      </c>
-      <c r="E5" s="14">
-        <f>metric!A5</f>
-        <v>22.859999965252801</v>
-      </c>
-      <c r="F5" s="15">
-        <f>metric!M5</f>
-        <v>2.56</v>
-      </c>
-      <c r="G5" s="14">
-        <f>metric!I5</f>
+      <c r="C70" s="15"/>
+      <c r="D70" s="15"/>
+      <c r="E70" s="15"/>
+      <c r="F70" s="15"/>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A71" s="15" cm="1">
+        <f t="array" ref="A71:B71">metric!I5:J5</f>
         <v>1.5239999976835199</v>
       </c>
-      <c r="H5" s="15">
-        <f>metric!J5</f>
+      <c r="B71" s="15">
         <v>1.23</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" s="14">
-        <f>metric!A24</f>
-        <v>109.72799983321345</v>
-      </c>
-      <c r="B6" s="15">
-        <f>metric!B24</f>
-        <v>2.99</v>
-      </c>
-      <c r="C6" s="14">
-        <f>metric!A24</f>
-        <v>109.72799983321345</v>
-      </c>
-      <c r="D6" s="15">
-        <f>metric!L24</f>
-        <v>3.0466666666666669</v>
-      </c>
-      <c r="E6" s="14">
-        <f>metric!A6</f>
-        <v>27.431999958303361</v>
-      </c>
-      <c r="F6" s="15">
-        <f>metric!M6</f>
-        <v>2.6199999999999997</v>
-      </c>
-      <c r="G6" s="14">
-        <f>metric!I6</f>
+      <c r="C71" s="15"/>
+      <c r="D71" s="15"/>
+      <c r="E71" s="15"/>
+      <c r="F71" s="15"/>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A72" s="15" cm="1">
+        <f t="array" ref="A72:B72">metric!I6:J6</f>
         <v>1.828799997220224</v>
       </c>
-      <c r="H6" s="15">
-        <f>metric!J6</f>
+      <c r="B72" s="15">
         <v>1.34</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A7" s="14">
-        <f>metric!A25</f>
-        <v>114.29999982626401</v>
-      </c>
-      <c r="B7" s="15">
-        <f>metric!B25</f>
-        <v>2.99</v>
-      </c>
-      <c r="C7" s="14">
-        <f>metric!A25</f>
-        <v>114.29999982626401</v>
-      </c>
-      <c r="D7" s="15">
-        <f>metric!L25</f>
-        <v>3.0533333333333332</v>
-      </c>
-      <c r="E7" s="14">
-        <f>metric!A7</f>
-        <v>32.003999951353926</v>
-      </c>
-      <c r="F7" s="15">
-        <f>metric!M7</f>
-        <v>2.6833333333333336</v>
-      </c>
-      <c r="G7" s="14">
-        <f>metric!I7</f>
+      <c r="C72" s="15"/>
+      <c r="D72" s="15"/>
+      <c r="E72" s="15"/>
+      <c r="F72" s="15"/>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A73" s="15" cm="1">
+        <f t="array" ref="A73:B73">metric!I7:J7</f>
         <v>2.1335999967569279</v>
       </c>
-      <c r="H7" s="15">
-        <f>metric!J7</f>
+      <c r="B73" s="15">
         <v>1.42</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" s="14">
-        <f>metric!A26</f>
-        <v>118.87199981931457</v>
-      </c>
-      <c r="B8" s="15">
-        <f>metric!B26</f>
-        <v>2.97</v>
-      </c>
-      <c r="C8" s="14">
-        <f>metric!A26</f>
-        <v>118.87199981931457</v>
-      </c>
-      <c r="D8" s="15">
-        <f>metric!L26</f>
-        <v>3.0666666666666664</v>
-      </c>
-      <c r="E8" s="14">
-        <f>metric!A8</f>
-        <v>36.575999944404487</v>
-      </c>
-      <c r="F8" s="15">
-        <f>metric!M8</f>
-        <v>2.7333333333333329</v>
-      </c>
-      <c r="G8" s="14">
-        <f>metric!I8</f>
+      <c r="C73" s="15"/>
+      <c r="D73" s="15"/>
+      <c r="E73" s="15"/>
+      <c r="F73" s="15"/>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A74" s="15" cm="1">
+        <f t="array" ref="A74:B74">metric!I8:J8</f>
         <v>2.438399996293632</v>
       </c>
-      <c r="H8" s="15">
-        <f>metric!J8</f>
+      <c r="B74" s="15">
         <v>1.5</v>
       </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" s="14">
-        <f>metric!A27</f>
-        <v>123.44399981236513</v>
-      </c>
-      <c r="B9" s="15">
-        <f>metric!B27</f>
-        <v>2.97</v>
-      </c>
-      <c r="C9" s="14">
-        <f>metric!A27</f>
-        <v>123.44399981236513</v>
-      </c>
-      <c r="D9" s="15">
-        <f>metric!L27</f>
-        <v>3.0833333333333335</v>
-      </c>
-      <c r="E9" s="14">
-        <f>metric!A9</f>
-        <v>41.147999937455047</v>
-      </c>
-      <c r="F9" s="15">
-        <f>metric!M9</f>
-        <v>2.78</v>
-      </c>
-      <c r="G9" s="14">
-        <f>metric!I9</f>
+      <c r="C74" s="15"/>
+      <c r="D74" s="15"/>
+      <c r="E74" s="15"/>
+      <c r="F74" s="15"/>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A75" s="15" cm="1">
+        <f t="array" ref="A75:B75">metric!I9:J9</f>
         <v>2.7431999958303357</v>
       </c>
-      <c r="H9" s="15">
-        <f>metric!J9</f>
+      <c r="B75" s="15">
         <v>1.56</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" s="14">
-        <f>metric!A28</f>
-        <v>128.0159998054157</v>
-      </c>
-      <c r="B10" s="15">
-        <f>metric!B28</f>
-        <v>2.97</v>
-      </c>
-      <c r="C10" s="14">
-        <f>metric!A28</f>
-        <v>128.0159998054157</v>
-      </c>
-      <c r="D10" s="15">
-        <f>metric!L28</f>
-        <v>3.0933333333333337</v>
-      </c>
-      <c r="E10" s="14">
-        <f>metric!A10</f>
-        <v>45.719999930505601</v>
-      </c>
-      <c r="F10" s="15">
-        <f>metric!M10</f>
-        <v>2.8266666666666667</v>
-      </c>
-      <c r="G10" s="14">
-        <f>metric!I10</f>
+      <c r="C75" s="15"/>
+      <c r="D75" s="15"/>
+      <c r="E75" s="15"/>
+      <c r="F75" s="15"/>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A76" s="15" cm="1">
+        <f t="array" ref="A76:B76">metric!I10:J10</f>
         <v>3.0479999953670398</v>
       </c>
-      <c r="H10" s="15">
-        <f>metric!J10</f>
+      <c r="B76" s="15">
         <v>1.61</v>
       </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A11" s="14">
-        <f>metric!A29</f>
-        <v>132.58799979846626</v>
-      </c>
-      <c r="B11" s="15">
-        <f>metric!B29</f>
-        <v>2.97</v>
-      </c>
-      <c r="C11" s="14">
-        <f>metric!A29</f>
-        <v>132.58799979846626</v>
-      </c>
-      <c r="D11" s="15">
-        <f>metric!L29</f>
-        <v>3.11</v>
-      </c>
-      <c r="E11" s="14">
-        <f>metric!A11</f>
-        <v>50.291999923556162</v>
-      </c>
-      <c r="F11" s="15">
-        <f>metric!M11</f>
-        <v>2.8733333333333331</v>
-      </c>
-      <c r="G11" s="14">
-        <f>metric!I11</f>
+      <c r="C76" s="15"/>
+      <c r="D76" s="15"/>
+      <c r="E76" s="15"/>
+      <c r="F76" s="15"/>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A77" s="15" cm="1">
+        <f t="array" ref="A77:B77">metric!I11:J11</f>
         <v>4.5719999930505599</v>
       </c>
-      <c r="H11" s="15">
-        <f>metric!J11</f>
+      <c r="B77" s="15">
         <v>1.78</v>
       </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12" s="14">
-        <f>metric!A30</f>
-        <v>137.15999979151681</v>
-      </c>
-      <c r="B12" s="15">
-        <f>metric!B30</f>
-        <v>2.99</v>
-      </c>
-      <c r="C12" s="14">
-        <f>metric!A30</f>
-        <v>137.15999979151681</v>
-      </c>
-      <c r="D12" s="15">
-        <f>metric!L30</f>
-        <v>3.1300000000000003</v>
-      </c>
-      <c r="E12" s="14">
-        <f>metric!A12</f>
-        <v>54.863999916606723</v>
-      </c>
-      <c r="F12" s="15">
-        <f>metric!M12</f>
-        <v>2.92</v>
-      </c>
-      <c r="G12" s="14">
-        <f>metric!I12</f>
+      <c r="C77" s="15"/>
+      <c r="D77" s="15"/>
+      <c r="E77" s="15"/>
+      <c r="F77" s="15"/>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78" s="15" cm="1">
+        <f t="array" ref="A78:B78">metric!I12:J12</f>
         <v>6.0959999907340796</v>
       </c>
-      <c r="H12" s="15">
-        <f>metric!J12</f>
+      <c r="B78" s="15">
         <v>1.87</v>
       </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A13" s="14">
-        <f>metric!A31</f>
-        <v>141.73199978456736</v>
-      </c>
-      <c r="B13" s="15">
-        <f>metric!B31</f>
-        <v>2.99</v>
-      </c>
-      <c r="C13" s="14">
-        <f>metric!A31</f>
-        <v>141.73199978456736</v>
-      </c>
-      <c r="D13" s="15">
-        <f>metric!L31</f>
-        <v>3.1466666666666665</v>
-      </c>
-      <c r="E13" s="14">
-        <f>metric!A13</f>
-        <v>59.435999909657284</v>
-      </c>
-      <c r="F13" s="15">
-        <f>metric!M13</f>
-        <v>2.936666666666667</v>
-      </c>
-      <c r="G13" s="14">
-        <f>metric!I13</f>
+      <c r="C78" s="15"/>
+      <c r="D78" s="15"/>
+      <c r="E78" s="15"/>
+      <c r="F78" s="15"/>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" s="15" cm="1">
+        <f t="array" ref="A79:B79">metric!I13:J13</f>
         <v>9.1439999861011199</v>
       </c>
-      <c r="H13" s="15">
-        <f>metric!J13</f>
+      <c r="B79" s="15">
         <v>1.98</v>
       </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A14" s="14">
-        <f>metric!A32</f>
-        <v>146.30399977761795</v>
-      </c>
-      <c r="B14" s="15">
-        <f>metric!B32</f>
-        <v>2.99</v>
-      </c>
-      <c r="C14" s="14">
-        <f>metric!A32</f>
-        <v>146.30399977761795</v>
-      </c>
-      <c r="D14" s="15">
-        <f>metric!L32</f>
-        <v>3.1633333333333336</v>
-      </c>
-      <c r="E14" s="14">
-        <f>metric!A14</f>
-        <v>64.007999902707851</v>
-      </c>
-      <c r="F14" s="15">
-        <f>metric!M14</f>
-        <v>2.9499999999999997</v>
-      </c>
-      <c r="G14" s="14">
-        <f>metric!I14</f>
+      <c r="C79" s="15"/>
+      <c r="D79" s="15"/>
+      <c r="E79" s="15"/>
+      <c r="F79" s="15"/>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A80" s="15" cm="1">
+        <f t="array" ref="A80:B80">metric!I14:J14</f>
         <v>12.191999981468159</v>
       </c>
-      <c r="H14" s="15">
-        <f>metric!J14</f>
+      <c r="B80" s="15">
         <v>2.06</v>
       </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A15" s="14">
-        <f>metric!A33</f>
-        <v>150.8759997706685</v>
-      </c>
-      <c r="B15" s="15">
-        <f>metric!B33</f>
-        <v>3.01</v>
-      </c>
-      <c r="C15" s="14">
-        <f>metric!A33</f>
-        <v>150.8759997706685</v>
-      </c>
-      <c r="D15" s="15">
-        <f>metric!L33</f>
-        <v>3.1833333333333336</v>
-      </c>
-      <c r="E15" s="14">
-        <f>metric!A15</f>
-        <v>68.579999895758405</v>
-      </c>
-      <c r="F15" s="15">
-        <f>metric!M15</f>
-        <v>2.97</v>
-      </c>
-      <c r="G15" s="14">
-        <f>metric!I15</f>
+      <c r="C80" s="15"/>
+      <c r="D80" s="15"/>
+      <c r="E80" s="15"/>
+      <c r="F80" s="15"/>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A81" s="15" cm="1">
+        <f t="array" ref="A81:B81">metric!I15:J15</f>
         <v>15.239999976835199</v>
       </c>
-      <c r="H15" s="15">
-        <f>metric!J15</f>
+      <c r="B81" s="15">
         <v>2.14</v>
       </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A16" s="14">
-        <f>metric!A34</f>
-        <v>155.44799976371905</v>
-      </c>
-      <c r="B16" s="15">
-        <f>metric!B34</f>
-        <v>3.02</v>
-      </c>
-      <c r="C16" s="14">
-        <f>metric!A34</f>
-        <v>155.44799976371905</v>
-      </c>
-      <c r="D16" s="15">
-        <f>metric!L34</f>
-        <v>3.2099999999999995</v>
-      </c>
-      <c r="E16" s="14">
-        <f>metric!A16</f>
-        <v>73.151999888808973</v>
-      </c>
-      <c r="F16" s="15">
-        <f>metric!M16</f>
-        <v>2.9833333333333329</v>
-      </c>
-      <c r="G16" s="14">
-        <f>metric!I16</f>
+      <c r="C81" s="15"/>
+      <c r="D81" s="15"/>
+      <c r="E81" s="15"/>
+      <c r="F81" s="15"/>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A82" s="15" cm="1">
+        <f t="array" ref="A82:B82">metric!I16:J16</f>
         <v>18.28799997220224</v>
       </c>
-      <c r="H16" s="15">
-        <f>metric!J16</f>
+      <c r="B82" s="15">
         <v>2.21</v>
       </c>
-    </row>
-    <row r="17" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="14">
-        <f>metric!A35</f>
-        <v>160.01999975676961</v>
-      </c>
-      <c r="B17" s="15">
-        <f>metric!B35</f>
-        <v>3.04</v>
-      </c>
-      <c r="C17" s="14">
-        <f>metric!A35</f>
-        <v>160.01999975676961</v>
-      </c>
-      <c r="D17" s="15">
-        <f>metric!L35</f>
-        <v>3.2366666666666664</v>
-      </c>
-      <c r="E17" s="14">
-        <f>metric!A17</f>
-        <v>77.723999881859527</v>
-      </c>
-      <c r="F17" s="15">
-        <f>metric!M17</f>
-        <v>2.9933333333333336</v>
-      </c>
-      <c r="G17" s="16">
-        <f>metric!I17</f>
+      <c r="C82" s="15"/>
+      <c r="D82" s="15"/>
+      <c r="E82" s="15"/>
+      <c r="F82" s="15"/>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A83" s="15" cm="1">
+        <f t="array" ref="A83:B83">metric!I17:J17</f>
         <v>27.431999958303358</v>
       </c>
-      <c r="H17" s="17">
-        <f>metric!J17</f>
+      <c r="B83" s="15">
         <v>2.4</v>
       </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A18" s="14">
-        <f>metric!A36</f>
-        <v>164.59199974982019</v>
-      </c>
-      <c r="B18" s="15">
-        <f>metric!B36</f>
-        <v>3.05</v>
-      </c>
-      <c r="C18" s="14">
-        <f>metric!A36</f>
-        <v>164.59199974982019</v>
-      </c>
-      <c r="D18" s="15">
-        <f>metric!L36</f>
-        <v>3.2633333333333336</v>
-      </c>
-      <c r="E18" s="14">
-        <f>metric!A18</f>
-        <v>82.295999874910095</v>
-      </c>
-      <c r="F18" s="15">
-        <f>metric!M18</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="14">
-        <f>metric!A37</f>
-        <v>169.16399974287074</v>
-      </c>
-      <c r="B19" s="15">
-        <f>metric!B37</f>
-        <v>3.07</v>
-      </c>
-      <c r="C19" s="14">
-        <f>metric!A37</f>
-        <v>169.16399974287074</v>
-      </c>
-      <c r="D19" s="15">
-        <f>metric!L37</f>
-        <v>3.293333333333333</v>
-      </c>
-      <c r="E19" s="16">
-        <f>metric!A19</f>
-        <v>86.867999867960648</v>
-      </c>
-      <c r="F19" s="17">
-        <f>metric!M19</f>
-        <v>3.01</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A20" s="14">
-        <f>metric!A38</f>
-        <v>173.7359997359213</v>
-      </c>
-      <c r="B20" s="15">
-        <f>metric!B38</f>
-        <v>3.09</v>
-      </c>
-      <c r="C20" s="14">
-        <f>metric!A38</f>
-        <v>173.7359997359213</v>
-      </c>
-      <c r="D20" s="15">
-        <f>metric!L38</f>
-        <v>3.3233333333333337</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A21" s="14">
-        <f>metric!A39</f>
-        <v>178.30799972897185</v>
-      </c>
-      <c r="B21" s="15">
-        <f>metric!B39</f>
-        <v>3.11</v>
-      </c>
-      <c r="C21" s="14">
-        <f>metric!A39</f>
-        <v>178.30799972897185</v>
-      </c>
-      <c r="D21" s="15">
-        <f>metric!L39</f>
-        <v>3.3566666666666669</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A22" s="14">
-        <f>metric!A40</f>
-        <v>182.8799997220224</v>
-      </c>
-      <c r="B22" s="15">
-        <f>metric!B40</f>
-        <v>3.12</v>
-      </c>
-      <c r="C22" s="14">
-        <f>metric!A40</f>
-        <v>182.8799997220224</v>
-      </c>
-      <c r="D22" s="15">
-        <f>metric!L40</f>
-        <v>3.3866666666666667</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A23" s="14">
-        <f>metric!A41</f>
-        <v>192.02399970812354</v>
-      </c>
-      <c r="B23" s="15">
-        <f>metric!B41</f>
-        <v>3.14</v>
-      </c>
-      <c r="C23" s="14">
-        <f>metric!A41</f>
-        <v>192.02399970812354</v>
-      </c>
-      <c r="D23" s="15">
-        <f>metric!L41</f>
-        <v>3.4533333333333331</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A24" s="14">
-        <f>metric!A42</f>
-        <v>201.16799969422465</v>
-      </c>
-      <c r="B24" s="15">
-        <f>metric!B42</f>
-        <v>3.17</v>
-      </c>
-      <c r="C24" s="14">
-        <f>metric!A42</f>
-        <v>201.16799969422465</v>
-      </c>
-      <c r="D24" s="15">
-        <f>metric!L42</f>
-        <v>3.5166666666666671</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A25" s="14">
-        <f>metric!A43</f>
-        <v>210.31199968032578</v>
-      </c>
-      <c r="B25" s="15">
-        <f>metric!B43</f>
-        <v>3.21</v>
-      </c>
-      <c r="C25" s="14">
-        <f>metric!A43</f>
-        <v>210.31199968032578</v>
-      </c>
-      <c r="D25" s="15">
-        <f>metric!L43</f>
-        <v>3.6533333333333329</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A26" s="14">
-        <f>metric!A44</f>
-        <v>219.45599966642689</v>
-      </c>
-      <c r="B26" s="15">
-        <f>metric!B44</f>
-        <v>3.25</v>
-      </c>
-      <c r="C26" s="14">
-        <f>metric!A44</f>
-        <v>219.45599966642689</v>
-      </c>
-      <c r="D26" s="15">
-        <f>metric!L44</f>
-        <v>3.6433333333333331</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A27" s="14">
-        <f>metric!A45</f>
-        <v>228.59999965252803</v>
-      </c>
-      <c r="B27" s="15">
-        <f>metric!B45</f>
-        <v>3.35</v>
-      </c>
-      <c r="C27" s="14">
-        <f>metric!A45</f>
-        <v>228.59999965252803</v>
-      </c>
-      <c r="D27" s="15">
-        <f>metric!L45</f>
-        <v>3.6966666666666668</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A28" s="14">
-        <f>metric!A46</f>
-        <v>237.74399963862913</v>
-      </c>
-      <c r="B28" s="15">
-        <f>metric!B46</f>
-        <v>3.45</v>
-      </c>
-      <c r="C28" s="14">
-        <f>metric!A46</f>
-        <v>237.74399963862913</v>
-      </c>
-      <c r="D28" s="15">
-        <f>metric!L46</f>
-        <v>3.75</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A29" s="14">
-        <f>metric!A47</f>
-        <v>246.88799962473027</v>
-      </c>
-      <c r="B29" s="15">
-        <f>metric!B47</f>
-        <v>3.55</v>
-      </c>
-      <c r="C29" s="14">
-        <f>metric!A47</f>
-        <v>246.88799962473027</v>
-      </c>
-      <c r="D29" s="15">
-        <f>metric!L47</f>
-        <v>3.7900000000000005</v>
-      </c>
-    </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A30" s="14">
-        <f>metric!A48</f>
-        <v>256.03199961083141</v>
-      </c>
-      <c r="B30" s="15">
-        <f>metric!B48</f>
-        <v>3.65</v>
-      </c>
-      <c r="C30" s="14">
-        <f>metric!A48</f>
-        <v>256.03199961083141</v>
-      </c>
-      <c r="D30" s="15">
-        <f>metric!L48</f>
-        <v>3.84</v>
-      </c>
-    </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A31" s="14">
-        <f>metric!A49</f>
-        <v>265.17599959693251</v>
-      </c>
-      <c r="B31" s="15">
-        <f>metric!B49</f>
-        <v>3.68</v>
-      </c>
-      <c r="C31" s="14">
-        <f>metric!A49</f>
-        <v>265.17599959693251</v>
-      </c>
-      <c r="D31" s="15">
-        <f>metric!L49</f>
-        <v>3.8766666666666665</v>
-      </c>
-    </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A32" s="14">
-        <f>metric!A50</f>
-        <v>274.31999958303362</v>
-      </c>
-      <c r="B32" s="15">
-        <f>metric!B50</f>
-        <v>3.71</v>
-      </c>
-      <c r="C32" s="14">
-        <f>metric!A50</f>
-        <v>274.31999958303362</v>
-      </c>
-      <c r="D32" s="15">
-        <f>metric!L50</f>
-        <v>3.9066666666666663</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33" s="14">
-        <f>metric!A51</f>
-        <v>292.60799955523589</v>
-      </c>
-      <c r="B33" s="15">
-        <f>metric!B51</f>
-        <v>3.79</v>
-      </c>
-      <c r="C33" s="14">
-        <f>metric!A51</f>
-        <v>292.60799955523589</v>
-      </c>
-      <c r="D33" s="15">
-        <f>metric!L51</f>
-        <v>3.97</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A34" s="14">
-        <f>metric!A52</f>
-        <v>310.89599952743811</v>
-      </c>
-      <c r="B34" s="15">
-        <f>metric!B52</f>
-        <v>3.86</v>
-      </c>
-      <c r="C34" s="14">
-        <f>metric!A52</f>
-        <v>310.89599952743811</v>
-      </c>
-      <c r="D34" s="15">
-        <f>metric!L52</f>
-        <v>4.0533333333333337</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A35" s="14">
-        <f>metric!A53</f>
-        <v>329.18399949964038</v>
-      </c>
-      <c r="B35" s="15">
-        <f>metric!B53</f>
-        <v>3.92</v>
-      </c>
-      <c r="C35" s="14">
-        <f>metric!A53</f>
-        <v>329.18399949964038</v>
-      </c>
-      <c r="D35" s="15">
-        <f>metric!L53</f>
-        <v>4.1566666666666672</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" s="14">
-        <f>metric!A54</f>
-        <v>347.47199947184259</v>
-      </c>
-      <c r="B36" s="15">
-        <f>metric!B54</f>
-        <v>3.96</v>
-      </c>
-      <c r="C36" s="14">
-        <f>metric!A54</f>
-        <v>347.47199947184259</v>
-      </c>
-      <c r="D36" s="15">
-        <f>metric!L54</f>
-        <v>4.2633333333333328</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A37" s="14">
-        <f>metric!A55</f>
-        <v>365.75999944404481</v>
-      </c>
-      <c r="B37" s="15">
-        <f>metric!B55</f>
-        <v>3.99</v>
-      </c>
-      <c r="C37" s="14">
-        <f>metric!A55</f>
-        <v>365.75999944404481</v>
-      </c>
-      <c r="D37" s="15">
-        <f>metric!L55</f>
-        <v>4.3666666666666671</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A38" s="14">
-        <f>metric!A56</f>
-        <v>384.04799941624708</v>
-      </c>
-      <c r="B38" s="15">
-        <f>metric!B56</f>
-        <v>4.0199999999999996</v>
-      </c>
-      <c r="C38" s="14">
-        <f>metric!A56</f>
-        <v>384.04799941624708</v>
-      </c>
-      <c r="D38" s="15">
-        <f>metric!L56</f>
-        <v>4.4066666666666672</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39" s="14">
-        <f>metric!A57</f>
-        <v>402.3359993884493</v>
-      </c>
-      <c r="B39" s="15">
-        <f>metric!B57</f>
-        <v>4.08</v>
-      </c>
-      <c r="C39" s="14">
-        <f>metric!A57</f>
-        <v>402.3359993884493</v>
-      </c>
-      <c r="D39" s="15">
-        <f>metric!L57</f>
-        <v>4.456666666666667</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40" s="14">
-        <f>metric!A58</f>
-        <v>420.62399936065157</v>
-      </c>
-      <c r="B40" s="15">
-        <f>metric!B58</f>
-        <v>4.17</v>
-      </c>
-      <c r="C40" s="14">
-        <f>metric!A58</f>
-        <v>420.62399936065157</v>
-      </c>
-      <c r="D40" s="15">
-        <f>metric!L58</f>
-        <v>4.5466666666666669</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41" s="14">
-        <f>metric!A59</f>
-        <v>438.91199933285378</v>
-      </c>
-      <c r="B41" s="15">
-        <f>metric!B59</f>
-        <v>4.28</v>
-      </c>
-      <c r="C41" s="14">
-        <f>metric!A59</f>
-        <v>438.91199933285378</v>
-      </c>
-      <c r="D41" s="15">
-        <f>metric!L59</f>
-        <v>4.6566666666666672</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42" s="14">
-        <f>metric!A60</f>
-        <v>457.19999930505605</v>
-      </c>
-      <c r="B42" s="15">
-        <f>metric!B60</f>
-        <v>4.41</v>
-      </c>
-      <c r="C42" s="14">
-        <f>metric!A60</f>
-        <v>457.19999930505605</v>
-      </c>
-      <c r="D42" s="15">
-        <f>metric!L60</f>
-        <v>4.7866666666666662</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A43" s="14">
-        <f>metric!A61</f>
-        <v>475.48799927725827</v>
-      </c>
-      <c r="B43" s="15">
-        <f>metric!B61</f>
-        <v>4.54</v>
-      </c>
-      <c r="C43" s="14">
-        <f>metric!A61</f>
-        <v>475.48799927725827</v>
-      </c>
-      <c r="D43" s="15">
-        <f>metric!L61</f>
-        <v>4.9799999999999995</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A44" s="14">
-        <f>metric!A62</f>
-        <v>493.77599924946054</v>
-      </c>
-      <c r="B44" s="15">
-        <f>metric!B62</f>
-        <v>4.6500000000000004</v>
-      </c>
-      <c r="C44" s="14">
-        <f>metric!A62</f>
-        <v>493.77599924946054</v>
-      </c>
-      <c r="D44" s="15">
-        <f>metric!L62</f>
-        <v>5.1000000000000005</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A45" s="14">
-        <f>metric!A63</f>
-        <v>512.06399922166281</v>
-      </c>
-      <c r="B45" s="15">
-        <f>metric!B63</f>
-        <v>4.74</v>
-      </c>
-      <c r="C45" s="14">
-        <f>metric!A63</f>
-        <v>512.06399922166281</v>
-      </c>
-      <c r="D45" s="15">
-        <f>metric!L63</f>
-        <v>5.18</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46" s="14">
-        <f>metric!A64</f>
-        <v>530.35199919386503</v>
-      </c>
-      <c r="B46" s="15">
-        <f>metric!B64</f>
-        <v>4.79</v>
-      </c>
-      <c r="C46" s="14">
-        <f>metric!A64</f>
-        <v>530.35199919386503</v>
-      </c>
-      <c r="D46" s="15">
-        <f>metric!L64</f>
-        <v>5.2299999999999995</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="16">
-        <f>metric!A65</f>
-        <v>548.63999916606724</v>
-      </c>
-      <c r="B47" s="17">
-        <f>metric!B65</f>
-        <v>4.82</v>
-      </c>
-      <c r="C47" s="16">
-        <f>metric!A65</f>
-        <v>548.63999916606724</v>
-      </c>
-      <c r="D47" s="17">
-        <f>metric!L65</f>
-        <v>5.26</v>
-      </c>
+      <c r="C83" s="15"/>
+      <c r="D83" s="15"/>
+      <c r="E83" s="15"/>
+      <c r="F83" s="15"/>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A84" s="15"/>
+      <c r="B84" s="15"/>
+      <c r="C84" s="15"/>
+      <c r="D84" s="15"/>
+      <c r="E84" s="15"/>
+      <c r="F84" s="15"/>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A85" s="15"/>
+      <c r="B85" s="15"/>
+      <c r="C85" s="15"/>
+      <c r="D85" s="15"/>
+      <c r="E85" s="15"/>
+      <c r="F85" s="15"/>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A86" s="15"/>
+      <c r="B86" s="15"/>
+      <c r="C86" s="15"/>
+      <c r="D86" s="15"/>
+      <c r="E86" s="15"/>
+      <c r="F86" s="15"/>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A87" s="15"/>
+      <c r="B87" s="15"/>
+      <c r="C87" s="15"/>
+      <c r="D87" s="15"/>
+      <c r="E87" s="15"/>
+      <c r="F87" s="15"/>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A88" s="15"/>
+      <c r="B88" s="15"/>
+      <c r="C88" s="15"/>
+      <c r="D88" s="15"/>
+      <c r="E88" s="15"/>
+      <c r="F88" s="15"/>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A89" s="15"/>
+      <c r="B89" s="15"/>
+      <c r="C89" s="15"/>
+      <c r="D89" s="15"/>
+      <c r="E89" s="15"/>
+      <c r="F89" s="15"/>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A90" s="15"/>
+      <c r="B90" s="15"/>
+      <c r="C90" s="15"/>
+      <c r="D90" s="15"/>
+      <c r="E90" s="15"/>
+      <c r="F90" s="15"/>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A91" s="15"/>
+      <c r="B91" s="15"/>
+      <c r="C91" s="15"/>
+      <c r="D91" s="15"/>
+      <c r="E91" s="15"/>
+      <c r="F91" s="15"/>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A92" s="15"/>
+      <c r="B92" s="15"/>
+      <c r="C92" s="15"/>
+      <c r="D92" s="15"/>
+      <c r="E92" s="15"/>
+      <c r="F92" s="15"/>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A93" s="15"/>
+      <c r="B93" s="15"/>
+      <c r="C93" s="15"/>
+      <c r="D93" s="15"/>
+      <c r="E93" s="15"/>
+      <c r="F93" s="15"/>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A94" s="15"/>
+      <c r="B94" s="15"/>
+      <c r="C94" s="15"/>
+      <c r="D94" s="15"/>
+      <c r="E94" s="15"/>
+      <c r="F94" s="15"/>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A95" s="15"/>
+      <c r="B95" s="15"/>
+      <c r="C95" s="15"/>
+      <c r="D95" s="15"/>
+      <c r="E95" s="15"/>
+      <c r="F95" s="15"/>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A96" s="15"/>
+      <c r="B96" s="15"/>
+      <c r="C96" s="15"/>
+      <c r="D96" s="15"/>
+      <c r="E96" s="15"/>
+      <c r="F96" s="15"/>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A97" s="15"/>
+      <c r="B97" s="15"/>
+      <c r="C97" s="15"/>
+      <c r="D97" s="15"/>
+      <c r="E97" s="15"/>
+      <c r="F97" s="15"/>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A98" s="15"/>
+      <c r="B98" s="15"/>
+      <c r="C98" s="15"/>
+      <c r="D98" s="15"/>
+      <c r="E98" s="15"/>
+      <c r="F98" s="15"/>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A99" s="15"/>
+      <c r="B99" s="15"/>
+      <c r="C99" s="15"/>
+      <c r="D99" s="15"/>
+      <c r="E99" s="15"/>
+      <c r="F99" s="15"/>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A100" s="15"/>
+      <c r="B100" s="15"/>
+      <c r="C100" s="15"/>
+      <c r="D100" s="15"/>
+      <c r="E100" s="15"/>
+      <c r="F100" s="15"/>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A101" s="15"/>
+      <c r="B101" s="15"/>
+      <c r="C101" s="15"/>
+      <c r="D101" s="15"/>
+      <c r="E101" s="15"/>
+      <c r="F101" s="15"/>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A102" s="15"/>
+      <c r="B102" s="15"/>
+      <c r="C102" s="15"/>
+      <c r="D102" s="15"/>
+      <c r="E102" s="15"/>
+      <c r="F102" s="15"/>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A103" s="15"/>
+      <c r="B103" s="15"/>
+      <c r="C103" s="15"/>
+      <c r="D103" s="15"/>
+      <c r="E103" s="15"/>
+      <c r="F103" s="15"/>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A104" s="15"/>
+      <c r="B104" s="15"/>
+      <c r="C104" s="15"/>
+      <c r="D104" s="15"/>
+      <c r="E104" s="15"/>
+      <c r="F104" s="15"/>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A105" s="15"/>
+      <c r="B105" s="15"/>
+      <c r="C105" s="15"/>
+      <c r="D105" s="15"/>
+      <c r="E105" s="15"/>
+      <c r="F105" s="15"/>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A106" s="15"/>
+      <c r="B106" s="15"/>
+      <c r="C106" s="15"/>
+      <c r="D106" s="15"/>
+      <c r="E106" s="15"/>
+      <c r="F106" s="15"/>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A107" s="15"/>
+      <c r="B107" s="15"/>
+      <c r="C107" s="15"/>
+      <c r="D107" s="15"/>
+      <c r="E107" s="15"/>
+      <c r="F107" s="15"/>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A108" s="15"/>
+      <c r="B108" s="15"/>
+      <c r="C108" s="15"/>
+      <c r="D108" s="15"/>
+      <c r="E108" s="15"/>
+      <c r="F108" s="15"/>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A109" s="15"/>
+      <c r="B109" s="15"/>
+      <c r="C109" s="15"/>
+      <c r="D109" s="15"/>
+      <c r="E109" s="15"/>
+      <c r="F109" s="15"/>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A110" s="15"/>
+      <c r="B110" s="15"/>
+      <c r="C110" s="15"/>
+      <c r="D110" s="15"/>
+      <c r="E110" s="15"/>
+      <c r="F110" s="15"/>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A111" s="15"/>
+      <c r="B111" s="15"/>
+      <c r="C111" s="15"/>
+      <c r="D111" s="15"/>
+      <c r="E111" s="15"/>
+      <c r="F111" s="15"/>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A112" s="15"/>
+      <c r="B112" s="15"/>
+      <c r="C112" s="15"/>
+      <c r="D112" s="15"/>
+      <c r="E112" s="15"/>
+      <c r="F112" s="15"/>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A113" s="15"/>
+      <c r="B113" s="15"/>
+      <c r="C113" s="15"/>
+      <c r="D113" s="15"/>
+      <c r="E113" s="15"/>
+      <c r="F113" s="15"/>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A114" s="15"/>
+      <c r="B114" s="15"/>
+      <c r="C114" s="15"/>
+      <c r="D114" s="15"/>
+      <c r="E114" s="15"/>
+      <c r="F114" s="15"/>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A115" s="15"/>
+      <c r="B115" s="15"/>
+      <c r="C115" s="15"/>
+      <c r="D115" s="15"/>
+      <c r="E115" s="15"/>
+      <c r="F115" s="15"/>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A116" s="15"/>
+      <c r="B116" s="15"/>
+      <c r="C116" s="15"/>
+      <c r="D116" s="15"/>
+      <c r="E116" s="15"/>
+      <c r="F116" s="15"/>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A117" s="15"/>
+      <c r="B117" s="15"/>
+      <c r="C117" s="15"/>
+      <c r="D117" s="15"/>
+      <c r="E117" s="15"/>
+      <c r="F117" s="15"/>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A118" s="15"/>
+      <c r="B118" s="15"/>
+      <c r="C118" s="15"/>
+      <c r="D118" s="15"/>
+      <c r="E118" s="15"/>
+      <c r="F118" s="15"/>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A119" s="15"/>
+      <c r="B119" s="15"/>
+      <c r="C119" s="15"/>
+      <c r="D119" s="15"/>
+      <c r="E119" s="15"/>
+      <c r="F119" s="15"/>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A120" s="15"/>
+      <c r="B120" s="15"/>
+      <c r="C120" s="15"/>
+      <c r="D120" s="15"/>
+      <c r="E120" s="15"/>
+      <c r="F120" s="15"/>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A121" s="15"/>
+      <c r="B121" s="15"/>
+      <c r="C121" s="15"/>
+      <c r="D121" s="15"/>
+      <c r="E121" s="15"/>
+      <c r="F121" s="15"/>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A122" s="15"/>
+      <c r="B122" s="15"/>
+      <c r="C122" s="15"/>
+      <c r="D122" s="15"/>
+      <c r="E122" s="15"/>
+      <c r="F122" s="15"/>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A123" s="15"/>
+      <c r="B123" s="15"/>
+      <c r="C123" s="15"/>
+      <c r="D123" s="15"/>
+      <c r="E123" s="15"/>
+      <c r="F123" s="15"/>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A124" s="15"/>
+      <c r="B124" s="15"/>
+      <c r="C124" s="15"/>
+      <c r="D124" s="15"/>
+      <c r="E124" s="15"/>
+      <c r="F124" s="15"/>
+    </row>
+    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A125" s="15"/>
+      <c r="B125" s="15"/>
+      <c r="C125" s="15"/>
+      <c r="D125" s="15"/>
+      <c r="E125" s="15"/>
+      <c r="F125" s="15"/>
+    </row>
+    <row r="126" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A126" s="15"/>
+      <c r="B126" s="15"/>
+      <c r="C126" s="15"/>
+      <c r="D126" s="15"/>
+      <c r="E126" s="15"/>
+      <c r="F126" s="15"/>
+    </row>
+    <row r="127" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A127" s="15"/>
+      <c r="B127" s="15"/>
+      <c r="C127" s="15"/>
+      <c r="D127" s="15"/>
+      <c r="E127" s="15"/>
+      <c r="F127" s="15"/>
+    </row>
+    <row r="128" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A128" s="15"/>
+      <c r="B128" s="15"/>
+      <c r="C128" s="15"/>
+      <c r="D128" s="15"/>
+      <c r="E128" s="15"/>
+      <c r="F128" s="15"/>
+    </row>
+    <row r="129" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A129" s="15"/>
+      <c r="B129" s="15"/>
+      <c r="C129" s="15"/>
+      <c r="D129" s="15"/>
+      <c r="E129" s="15"/>
+      <c r="F129" s="15"/>
+    </row>
+    <row r="130" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A130" s="15"/>
+      <c r="B130" s="15"/>
+      <c r="C130" s="15"/>
+      <c r="D130" s="15"/>
+      <c r="E130" s="15"/>
+      <c r="F130" s="15"/>
+    </row>
+    <row r="131" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A131" s="15"/>
+      <c r="B131" s="15"/>
+      <c r="C131" s="15"/>
+      <c r="D131" s="15"/>
+      <c r="E131" s="15"/>
+      <c r="F131" s="15"/>
+    </row>
+    <row r="132" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A132" s="15"/>
+      <c r="B132" s="15"/>
+      <c r="C132" s="15"/>
+      <c r="D132" s="15"/>
+      <c r="E132" s="15"/>
+      <c r="F132" s="15"/>
+    </row>
+    <row r="133" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A133" s="15"/>
+      <c r="B133" s="15"/>
+      <c r="C133" s="15"/>
+      <c r="D133" s="15"/>
+      <c r="E133" s="15"/>
+      <c r="F133" s="15"/>
+    </row>
+    <row r="134" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A134" s="15"/>
+      <c r="B134" s="15"/>
+      <c r="C134" s="15"/>
+      <c r="D134" s="15"/>
+      <c r="E134" s="15"/>
+      <c r="F134" s="15"/>
+    </row>
+    <row r="135" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A135" s="15"/>
+      <c r="B135" s="15"/>
+      <c r="C135" s="15"/>
+      <c r="D135" s="15"/>
+      <c r="E135" s="15"/>
+      <c r="F135" s="15"/>
+    </row>
+    <row r="136" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A136" s="15"/>
+      <c r="B136" s="15"/>
+      <c r="C136" s="15"/>
+      <c r="D136" s="15"/>
+      <c r="E136" s="15"/>
+      <c r="F136" s="15"/>
+    </row>
+    <row r="137" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A137" s="15"/>
+      <c r="B137" s="15"/>
+      <c r="C137" s="15"/>
+      <c r="D137" s="15"/>
+      <c r="E137" s="15"/>
+      <c r="F137" s="15"/>
+    </row>
+    <row r="138" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A138" s="15"/>
+      <c r="B138" s="15"/>
+      <c r="C138" s="15"/>
+      <c r="D138" s="15"/>
+      <c r="E138" s="15"/>
+      <c r="F138" s="15"/>
+    </row>
+    <row r="139" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A139" s="15"/>
+      <c r="B139" s="15"/>
+      <c r="C139" s="15"/>
+      <c r="D139" s="15"/>
+      <c r="E139" s="15"/>
+      <c r="F139" s="15"/>
+    </row>
+    <row r="140" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A140" s="15"/>
+      <c r="B140" s="15"/>
+      <c r="C140" s="15"/>
+      <c r="D140" s="15"/>
+      <c r="E140" s="15"/>
+      <c r="F140" s="15"/>
+    </row>
+    <row r="141" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A141" s="15"/>
+      <c r="B141" s="15"/>
+      <c r="C141" s="15"/>
+      <c r="D141" s="15"/>
+      <c r="E141" s="15"/>
+      <c r="F141" s="15"/>
+    </row>
+    <row r="142" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A142" s="15"/>
+      <c r="B142" s="15"/>
+      <c r="C142" s="15"/>
+      <c r="D142" s="15"/>
+      <c r="E142" s="15"/>
+      <c r="F142" s="15"/>
+    </row>
+    <row r="143" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A143" s="15"/>
+      <c r="B143" s="15"/>
+      <c r="C143" s="15"/>
+      <c r="D143" s="15"/>
+      <c r="E143" s="15"/>
+      <c r="F143" s="15"/>
+    </row>
+    <row r="144" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A144" s="15"/>
+      <c r="B144" s="15"/>
+      <c r="C144" s="15"/>
+      <c r="D144" s="15"/>
+      <c r="E144" s="15"/>
+      <c r="F144" s="15"/>
+    </row>
+    <row r="145" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A145" s="15"/>
+      <c r="B145" s="15"/>
+      <c r="C145" s="15"/>
+      <c r="D145" s="15"/>
+      <c r="E145" s="15"/>
+      <c r="F145" s="15"/>
+    </row>
+    <row r="146" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A146" s="15"/>
+      <c r="B146" s="15"/>
+      <c r="C146" s="15"/>
+      <c r="D146" s="15"/>
+      <c r="E146" s="15"/>
+      <c r="F146" s="15"/>
+    </row>
+    <row r="147" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A147" s="15"/>
+      <c r="B147" s="15"/>
+      <c r="C147" s="15"/>
+      <c r="D147" s="15"/>
+      <c r="E147" s="15"/>
+      <c r="F147" s="15"/>
+    </row>
+    <row r="148" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A148" s="15"/>
+      <c r="B148" s="15"/>
+      <c r="C148" s="15"/>
+      <c r="D148" s="15"/>
+      <c r="E148" s="15"/>
+      <c r="F148" s="15"/>
+    </row>
+    <row r="149" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A149" s="15"/>
+      <c r="B149" s="15"/>
+      <c r="C149" s="15"/>
+      <c r="D149" s="15"/>
+      <c r="E149" s="15"/>
+      <c r="F149" s="15"/>
+    </row>
+    <row r="150" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A150" s="15"/>
+      <c r="B150" s="15"/>
+      <c r="C150" s="15"/>
+      <c r="D150" s="15"/>
+      <c r="E150" s="15"/>
+      <c r="F150" s="15"/>
+    </row>
+    <row r="151" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A151" s="15"/>
+      <c r="B151" s="15"/>
+      <c r="C151" s="15"/>
+      <c r="D151" s="15"/>
+      <c r="E151" s="15"/>
+      <c r="F151" s="15"/>
+    </row>
+    <row r="152" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A152" s="15"/>
+      <c r="B152" s="15"/>
+      <c r="C152" s="15"/>
+      <c r="D152" s="15"/>
+      <c r="E152" s="15"/>
+      <c r="F152" s="15"/>
+    </row>
+    <row r="153" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A153" s="15"/>
+      <c r="B153" s="15"/>
+      <c r="C153" s="15"/>
+      <c r="D153" s="15"/>
+      <c r="E153" s="15"/>
+      <c r="F153" s="15"/>
+    </row>
+    <row r="154" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A154" s="15"/>
+      <c r="B154" s="15"/>
+      <c r="C154" s="15"/>
+      <c r="D154" s="15"/>
+      <c r="E154" s="15"/>
+      <c r="F154" s="15"/>
+    </row>
+    <row r="155" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A155" s="15"/>
+      <c r="B155" s="15"/>
+      <c r="C155" s="15"/>
+      <c r="D155" s="15"/>
+      <c r="E155" s="15"/>
+      <c r="F155" s="15"/>
+    </row>
+    <row r="156" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A156" s="15"/>
+      <c r="B156" s="15"/>
+      <c r="C156" s="15"/>
+      <c r="D156" s="15"/>
+      <c r="E156" s="15"/>
+      <c r="F156" s="15"/>
+    </row>
+    <row r="157" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A157" s="15"/>
+      <c r="B157" s="15"/>
+      <c r="C157" s="15"/>
+      <c r="D157" s="15"/>
+      <c r="E157" s="15"/>
+      <c r="F157" s="15"/>
+    </row>
+    <row r="158" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A158" s="15"/>
+      <c r="B158" s="15"/>
+      <c r="C158" s="15"/>
+      <c r="D158" s="15"/>
+      <c r="E158" s="15"/>
+      <c r="F158" s="15"/>
+    </row>
+    <row r="159" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A159" s="15"/>
+      <c r="B159" s="15"/>
+      <c r="C159" s="15"/>
+      <c r="D159" s="15"/>
+      <c r="E159" s="15"/>
+      <c r="F159" s="15"/>
+    </row>
+    <row r="160" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A160" s="15"/>
+      <c r="B160" s="15"/>
+      <c r="C160" s="15"/>
+      <c r="D160" s="15"/>
+      <c r="E160" s="15"/>
+      <c r="F160" s="15"/>
+    </row>
+    <row r="161" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A161" s="15"/>
+      <c r="B161" s="15"/>
+      <c r="C161" s="15"/>
+      <c r="D161" s="15"/>
+      <c r="E161" s="15"/>
+      <c r="F161" s="15"/>
+    </row>
+    <row r="162" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A162" s="15"/>
+      <c r="B162" s="15"/>
+      <c r="C162" s="15"/>
+      <c r="D162" s="15"/>
+      <c r="E162" s="15"/>
+      <c r="F162" s="15"/>
+    </row>
+    <row r="163" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A163" s="15"/>
+      <c r="B163" s="15"/>
+      <c r="C163" s="15"/>
+      <c r="D163" s="15"/>
+      <c r="E163" s="15"/>
+      <c r="F163" s="15"/>
+    </row>
+    <row r="164" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A164" s="15"/>
+      <c r="B164" s="15"/>
+      <c r="C164" s="15"/>
+      <c r="D164" s="15"/>
+      <c r="E164" s="15"/>
+      <c r="F164" s="15"/>
+    </row>
+    <row r="165" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A165" s="15"/>
+      <c r="B165" s="15"/>
+      <c r="C165" s="15"/>
+      <c r="D165" s="15"/>
+      <c r="E165" s="15"/>
+      <c r="F165" s="15"/>
+    </row>
+    <row r="166" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A166" s="15"/>
+      <c r="B166" s="15"/>
+      <c r="C166" s="15"/>
+      <c r="D166" s="15"/>
+      <c r="E166" s="15"/>
+      <c r="F166" s="15"/>
+    </row>
+    <row r="167" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A167" s="15"/>
+      <c r="B167" s="15"/>
+      <c r="C167" s="15"/>
+      <c r="D167" s="15"/>
+      <c r="E167" s="15"/>
+      <c r="F167" s="15"/>
+    </row>
+    <row r="168" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A168" s="15"/>
+      <c r="B168" s="15"/>
+      <c r="C168" s="15"/>
+      <c r="D168" s="15"/>
+      <c r="E168" s="15"/>
+      <c r="F168" s="15"/>
+    </row>
+    <row r="169" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A169" s="15"/>
+      <c r="B169" s="15"/>
+      <c r="C169" s="15"/>
+      <c r="D169" s="15"/>
+      <c r="E169" s="15"/>
+      <c r="F169" s="15"/>
+    </row>
+    <row r="170" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A170" s="15"/>
+      <c r="B170" s="15"/>
+      <c r="C170" s="15"/>
+      <c r="D170" s="15"/>
+      <c r="E170" s="15"/>
+      <c r="F170" s="15"/>
+    </row>
+    <row r="171" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A171" s="15"/>
+      <c r="B171" s="15"/>
+      <c r="C171" s="15"/>
+      <c r="D171" s="15"/>
+      <c r="E171" s="15"/>
+      <c r="F171" s="15"/>
+    </row>
+    <row r="172" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A172" s="15"/>
+      <c r="B172" s="15"/>
+      <c r="C172" s="15"/>
+      <c r="D172" s="15"/>
+      <c r="E172" s="15"/>
+      <c r="F172" s="15"/>
+    </row>
+    <row r="173" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A173" s="15"/>
+      <c r="B173" s="15"/>
+      <c r="C173" s="15"/>
+      <c r="D173" s="15"/>
+      <c r="E173" s="15"/>
+      <c r="F173" s="15"/>
+    </row>
+    <row r="174" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A174" s="15"/>
+      <c r="B174" s="15"/>
+      <c r="C174" s="15"/>
+      <c r="D174" s="15"/>
+      <c r="E174" s="15"/>
+      <c r="F174" s="15"/>
+    </row>
+    <row r="175" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A175" s="15"/>
+      <c r="B175" s="15"/>
+      <c r="C175" s="15"/>
+      <c r="D175" s="15"/>
+      <c r="E175" s="15"/>
+      <c r="F175" s="15"/>
+    </row>
+    <row r="176" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A176" s="15"/>
+      <c r="B176" s="15"/>
+      <c r="C176" s="15"/>
+      <c r="D176" s="15"/>
+      <c r="E176" s="15"/>
+      <c r="F176" s="15"/>
+    </row>
+    <row r="177" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A177" s="15"/>
+      <c r="B177" s="15"/>
+      <c r="C177" s="15"/>
+      <c r="D177" s="15"/>
+      <c r="E177" s="15"/>
+      <c r="F177" s="15"/>
+    </row>
+    <row r="178" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A178" s="15"/>
+      <c r="B178" s="15"/>
+      <c r="C178" s="15"/>
+      <c r="D178" s="15"/>
+      <c r="E178" s="15"/>
+      <c r="F178" s="15"/>
+    </row>
+    <row r="179" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A179" s="15"/>
+      <c r="B179" s="15"/>
+      <c r="C179" s="15"/>
+      <c r="D179" s="15"/>
+      <c r="E179" s="15"/>
+      <c r="F179" s="15"/>
+    </row>
+    <row r="180" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A180" s="15"/>
+      <c r="B180" s="15"/>
+      <c r="C180" s="15"/>
+      <c r="D180" s="15"/>
+      <c r="E180" s="15"/>
+      <c r="F180" s="15"/>
+    </row>
+    <row r="181" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A181" s="15"/>
+      <c r="B181" s="15"/>
+      <c r="C181" s="15"/>
+      <c r="D181" s="15"/>
+      <c r="E181" s="15"/>
+      <c r="F181" s="15"/>
+    </row>
+    <row r="182" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A182" s="15"/>
+      <c r="B182" s="15"/>
+      <c r="C182" s="15"/>
+      <c r="D182" s="15"/>
+      <c r="E182" s="15"/>
+      <c r="F182" s="15"/>
+    </row>
+    <row r="183" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A183" s="15"/>
+      <c r="B183" s="15"/>
+      <c r="C183" s="15"/>
+      <c r="D183" s="15"/>
+      <c r="E183" s="15"/>
+      <c r="F183" s="15"/>
+    </row>
+    <row r="184" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A184" s="15"/>
+      <c r="B184" s="15"/>
+      <c r="C184" s="15"/>
+      <c r="D184" s="15"/>
+      <c r="E184" s="15"/>
+      <c r="F184" s="15"/>
+    </row>
+    <row r="185" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A185" s="15"/>
+      <c r="B185" s="15"/>
+      <c r="C185" s="15"/>
+      <c r="D185" s="15"/>
+      <c r="E185" s="15"/>
+      <c r="F185" s="15"/>
+    </row>
+    <row r="186" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A186" s="15"/>
+      <c r="B186" s="15"/>
+      <c r="C186" s="15"/>
+      <c r="D186" s="15"/>
+      <c r="E186" s="15"/>
+      <c r="F186" s="15"/>
+    </row>
+    <row r="187" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A187" s="15"/>
+      <c r="B187" s="15"/>
+      <c r="C187" s="15"/>
+      <c r="D187" s="15"/>
+      <c r="E187" s="15"/>
+      <c r="F187" s="15"/>
+    </row>
+    <row r="188" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A188" s="15"/>
+      <c r="B188" s="15"/>
+      <c r="C188" s="15"/>
+      <c r="D188" s="15"/>
+      <c r="E188" s="15"/>
+      <c r="F188" s="15"/>
+    </row>
+    <row r="189" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A189" s="15"/>
+      <c r="B189" s="15"/>
+      <c r="C189" s="15"/>
+      <c r="D189" s="15"/>
+      <c r="E189" s="15"/>
+      <c r="F189" s="15"/>
+    </row>
+    <row r="190" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A190" s="15"/>
+      <c r="B190" s="15"/>
+      <c r="C190" s="15"/>
+      <c r="D190" s="15"/>
+      <c r="E190" s="15"/>
+      <c r="F190" s="15"/>
+    </row>
+    <row r="191" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A191" s="15"/>
+      <c r="B191" s="15"/>
+      <c r="C191" s="15"/>
+      <c r="D191" s="15"/>
+      <c r="E191" s="15"/>
+      <c r="F191" s="15"/>
+    </row>
+    <row r="192" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A192" s="15"/>
+      <c r="B192" s="15"/>
+      <c r="C192" s="15"/>
+      <c r="D192" s="15"/>
+      <c r="E192" s="15"/>
+      <c r="F192" s="15"/>
+    </row>
+    <row r="193" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A193" s="15"/>
+      <c r="B193" s="15"/>
+      <c r="C193" s="15"/>
+      <c r="D193" s="15"/>
+      <c r="E193" s="15"/>
+      <c r="F193" s="15"/>
+    </row>
+    <row r="194" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A194" s="15"/>
+      <c r="B194" s="15"/>
+      <c r="C194" s="15"/>
+      <c r="D194" s="15"/>
+      <c r="E194" s="15"/>
+      <c r="F194" s="15"/>
+    </row>
+    <row r="195" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A195" s="15"/>
+      <c r="B195" s="15"/>
+      <c r="C195" s="15"/>
+      <c r="D195" s="15"/>
+      <c r="E195" s="15"/>
+      <c r="F195" s="15"/>
+    </row>
+    <row r="196" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A196" s="15"/>
+      <c r="B196" s="15"/>
+      <c r="C196" s="15"/>
+      <c r="D196" s="15"/>
+      <c r="E196" s="15"/>
+      <c r="F196" s="15"/>
+    </row>
+    <row r="197" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A197" s="15"/>
+      <c r="B197" s="15"/>
+      <c r="C197" s="15"/>
+      <c r="D197" s="15"/>
+      <c r="E197" s="15"/>
+      <c r="F197" s="15"/>
+    </row>
+    <row r="198" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A198" s="15"/>
+      <c r="B198" s="15"/>
+      <c r="C198" s="15"/>
+      <c r="D198" s="15"/>
+      <c r="E198" s="15"/>
+      <c r="F198" s="15"/>
+    </row>
+    <row r="199" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A199" s="15"/>
+      <c r="B199" s="15"/>
+      <c r="C199" s="15"/>
+      <c r="D199" s="15"/>
+      <c r="E199" s="15"/>
+      <c r="F199" s="15"/>
+    </row>
+    <row r="200" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A200" s="15"/>
+      <c r="B200" s="15"/>
+      <c r="C200" s="15"/>
+      <c r="D200" s="15"/>
+      <c r="E200" s="15"/>
+      <c r="F200" s="15"/>
+    </row>
+    <row r="201" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A201" s="15"/>
+      <c r="B201" s="15"/>
+      <c r="C201" s="15"/>
+      <c r="D201" s="15"/>
+      <c r="E201" s="15"/>
+      <c r="F201" s="15"/>
+    </row>
+    <row r="202" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A202" s="15"/>
+      <c r="B202" s="15"/>
+      <c r="C202" s="15"/>
+      <c r="D202" s="15"/>
+      <c r="E202" s="15"/>
+      <c r="F202" s="15"/>
+    </row>
+    <row r="203" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A203" s="15"/>
+      <c r="B203" s="15"/>
+      <c r="C203" s="15"/>
+      <c r="D203" s="15"/>
+      <c r="E203" s="15"/>
+      <c r="F203" s="15"/>
+    </row>
+    <row r="204" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A204" s="15"/>
+      <c r="B204" s="15"/>
+      <c r="C204" s="15"/>
+      <c r="D204" s="15"/>
+      <c r="E204" s="15"/>
+      <c r="F204" s="15"/>
+    </row>
+    <row r="205" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A205" s="15"/>
+      <c r="B205" s="15"/>
+      <c r="C205" s="15"/>
+      <c r="D205" s="15"/>
+      <c r="E205" s="15"/>
+      <c r="F205" s="15"/>
+    </row>
+    <row r="206" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A206" s="15"/>
+      <c r="B206" s="15"/>
+      <c r="C206" s="15"/>
+      <c r="D206" s="15"/>
+      <c r="E206" s="15"/>
+      <c r="F206" s="15"/>
+    </row>
+    <row r="207" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A207" s="15"/>
+      <c r="B207" s="15"/>
+      <c r="C207" s="15"/>
+      <c r="D207" s="15"/>
+      <c r="E207" s="15"/>
+      <c r="F207" s="15"/>
+    </row>
+    <row r="208" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A208" s="15"/>
+      <c r="B208" s="15"/>
+      <c r="C208" s="15"/>
+      <c r="D208" s="15"/>
+      <c r="E208" s="15"/>
+      <c r="F208" s="15"/>
+    </row>
+    <row r="209" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A209" s="15"/>
+      <c r="B209" s="15"/>
+      <c r="C209" s="15"/>
+      <c r="D209" s="15"/>
+      <c r="E209" s="15"/>
+      <c r="F209" s="15"/>
+    </row>
+    <row r="210" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A210" s="15"/>
+      <c r="B210" s="15"/>
+      <c r="C210" s="15"/>
+      <c r="D210" s="15"/>
+      <c r="E210" s="15"/>
+      <c r="F210" s="15"/>
+    </row>
+    <row r="211" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A211" s="15"/>
+      <c r="B211" s="15"/>
+      <c r="C211" s="15"/>
+      <c r="D211" s="15"/>
+      <c r="E211" s="15"/>
+      <c r="F211" s="15"/>
+    </row>
+    <row r="212" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A212" s="15"/>
+      <c r="B212" s="15"/>
+      <c r="C212" s="15"/>
+      <c r="D212" s="15"/>
+      <c r="E212" s="15"/>
+      <c r="F212" s="15"/>
+    </row>
+    <row r="213" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A213" s="15"/>
+      <c r="B213" s="15"/>
+      <c r="C213" s="15"/>
+      <c r="D213" s="15"/>
+      <c r="E213" s="15"/>
+      <c r="F213" s="15"/>
+    </row>
+    <row r="214" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A214" s="15"/>
+      <c r="B214" s="15"/>
+      <c r="C214" s="15"/>
+      <c r="D214" s="15"/>
+      <c r="E214" s="15"/>
+      <c r="F214" s="15"/>
+    </row>
+    <row r="215" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A215" s="15"/>
+      <c r="B215" s="15"/>
+      <c r="C215" s="15"/>
+      <c r="D215" s="15"/>
+      <c r="E215" s="15"/>
+      <c r="F215" s="15"/>
+    </row>
+    <row r="216" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A216" s="15"/>
+      <c r="B216" s="15"/>
+      <c r="C216" s="15"/>
+      <c r="D216" s="15"/>
+      <c r="E216" s="15"/>
+      <c r="F216" s="15"/>
+    </row>
+    <row r="217" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A217" s="15"/>
+      <c r="B217" s="15"/>
+      <c r="C217" s="15"/>
+      <c r="D217" s="15"/>
+      <c r="E217" s="15"/>
+      <c r="F217" s="15"/>
+    </row>
+    <row r="218" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A218" s="15"/>
+      <c r="B218" s="15"/>
+      <c r="C218" s="15"/>
+      <c r="D218" s="15"/>
+      <c r="E218" s="15"/>
+      <c r="F218" s="15"/>
+    </row>
+    <row r="219" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A219" s="15"/>
+      <c r="B219" s="15"/>
+      <c r="C219" s="15"/>
+      <c r="D219" s="15"/>
+      <c r="E219" s="15"/>
+      <c r="F219" s="15"/>
+    </row>
+    <row r="220" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A220" s="15"/>
+      <c r="B220" s="15"/>
+      <c r="C220" s="15"/>
+      <c r="D220" s="15"/>
+      <c r="E220" s="15"/>
+      <c r="F220" s="15"/>
+    </row>
+    <row r="221" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A221" s="15"/>
+      <c r="B221" s="15"/>
+      <c r="C221" s="15"/>
+      <c r="D221" s="15"/>
+      <c r="E221" s="15"/>
+      <c r="F221" s="15"/>
+    </row>
+    <row r="222" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A222" s="15"/>
+      <c r="B222" s="15"/>
+      <c r="C222" s="15"/>
+      <c r="D222" s="15"/>
+      <c r="E222" s="15"/>
+      <c r="F222" s="15"/>
+    </row>
+    <row r="223" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A223" s="15"/>
+      <c r="B223" s="15"/>
+      <c r="C223" s="15"/>
+      <c r="D223" s="15"/>
+      <c r="E223" s="15"/>
+      <c r="F223" s="15"/>
+    </row>
+    <row r="224" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A224" s="15"/>
+      <c r="B224" s="15"/>
+      <c r="C224" s="15"/>
+      <c r="D224" s="15"/>
+      <c r="E224" s="15"/>
+      <c r="F224" s="15"/>
+    </row>
+    <row r="225" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A225" s="15"/>
+      <c r="B225" s="15"/>
+      <c r="C225" s="15"/>
+      <c r="D225" s="15"/>
+      <c r="E225" s="15"/>
+      <c r="F225" s="15"/>
+    </row>
+    <row r="226" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A226" s="15"/>
+      <c r="B226" s="15"/>
+      <c r="C226" s="15"/>
+      <c r="D226" s="15"/>
+      <c r="E226" s="15"/>
+      <c r="F226" s="15"/>
+    </row>
+    <row r="227" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A227" s="15"/>
+      <c r="B227" s="15"/>
+      <c r="C227" s="15"/>
+      <c r="D227" s="15"/>
+      <c r="E227" s="15"/>
+      <c r="F227" s="15"/>
+    </row>
+    <row r="228" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A228" s="15"/>
+      <c r="B228" s="15"/>
+      <c r="C228" s="15"/>
+      <c r="D228" s="15"/>
+      <c r="E228" s="15"/>
+      <c r="F228" s="15"/>
+    </row>
+    <row r="229" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A229" s="15"/>
+      <c r="B229" s="15"/>
+      <c r="C229" s="15"/>
+      <c r="D229" s="15"/>
+      <c r="E229" s="15"/>
+      <c r="F229" s="15"/>
+    </row>
+    <row r="230" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A230" s="15"/>
+      <c r="B230" s="15"/>
+      <c r="C230" s="15"/>
+      <c r="D230" s="15"/>
+      <c r="E230" s="15"/>
+      <c r="F230" s="15"/>
+    </row>
+    <row r="231" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A231" s="15"/>
+      <c r="B231" s="15"/>
+      <c r="C231" s="15"/>
+      <c r="D231" s="15"/>
+      <c r="E231" s="15"/>
+      <c r="F231" s="15"/>
+    </row>
+    <row r="232" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A232" s="15"/>
+      <c r="B232" s="15"/>
+      <c r="C232" s="15"/>
+      <c r="D232" s="15"/>
+      <c r="E232" s="15"/>
+      <c r="F232" s="15"/>
+    </row>
+    <row r="233" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A233" s="15"/>
+      <c r="B233" s="15"/>
+      <c r="C233" s="15"/>
+      <c r="D233" s="15"/>
+      <c r="E233" s="15"/>
+      <c r="F233" s="15"/>
+    </row>
+    <row r="234" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A234" s="15"/>
+      <c r="B234" s="15"/>
+      <c r="C234" s="15"/>
+      <c r="D234" s="15"/>
+      <c r="E234" s="15"/>
+      <c r="F234" s="15"/>
+    </row>
+    <row r="235" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A235" s="15"/>
+      <c r="B235" s="15"/>
+      <c r="C235" s="15"/>
+      <c r="D235" s="15"/>
+      <c r="E235" s="15"/>
+      <c r="F235" s="15"/>
+    </row>
+    <row r="236" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A236" s="15"/>
+      <c r="B236" s="15"/>
+      <c r="C236" s="15"/>
+      <c r="D236" s="15"/>
+      <c r="E236" s="15"/>
+      <c r="F236" s="15"/>
+    </row>
+    <row r="237" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A237" s="15"/>
+      <c r="B237" s="15"/>
+      <c r="C237" s="15"/>
+      <c r="D237" s="15"/>
+      <c r="E237" s="15"/>
+      <c r="F237" s="15"/>
+    </row>
+    <row r="238" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A238" s="15"/>
+      <c r="B238" s="15"/>
+      <c r="C238" s="15"/>
+      <c r="D238" s="15"/>
+      <c r="E238" s="15"/>
+      <c r="F238" s="15"/>
+    </row>
+    <row r="239" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A239" s="15"/>
+      <c r="B239" s="15"/>
+      <c r="C239" s="15"/>
+      <c r="D239" s="15"/>
+      <c r="E239" s="15"/>
+      <c r="F239" s="15"/>
+    </row>
+    <row r="240" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A240" s="15"/>
+      <c r="B240" s="15"/>
+      <c r="C240" s="15"/>
+      <c r="D240" s="15"/>
+      <c r="E240" s="15"/>
+      <c r="F240" s="15"/>
+    </row>
+    <row r="241" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A241" s="15"/>
+      <c r="B241" s="15"/>
+      <c r="C241" s="15"/>
+      <c r="D241" s="15"/>
+      <c r="E241" s="15"/>
+      <c r="F241" s="15"/>
+    </row>
+    <row r="242" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A242" s="15"/>
+      <c r="B242" s="15"/>
+      <c r="C242" s="15"/>
+      <c r="D242" s="15"/>
+      <c r="E242" s="15"/>
+      <c r="F242" s="15"/>
+    </row>
+    <row r="243" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A243" s="15"/>
+      <c r="B243" s="15"/>
+      <c r="C243" s="15"/>
+      <c r="D243" s="15"/>
+      <c r="E243" s="15"/>
+      <c r="F243" s="15"/>
+    </row>
+    <row r="244" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A244" s="15"/>
+      <c r="B244" s="15"/>
+      <c r="C244" s="15"/>
+      <c r="D244" s="15"/>
+      <c r="E244" s="15"/>
+      <c r="F244" s="15"/>
+    </row>
+    <row r="245" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A245" s="15"/>
+      <c r="B245" s="15"/>
+      <c r="C245" s="15"/>
+      <c r="D245" s="15"/>
+      <c r="E245" s="15"/>
+      <c r="F245" s="15"/>
+    </row>
+    <row r="246" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A246" s="15"/>
+      <c r="B246" s="15"/>
+      <c r="C246" s="15"/>
+      <c r="D246" s="15"/>
+      <c r="E246" s="15"/>
+      <c r="F246" s="15"/>
+    </row>
+    <row r="247" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A247" s="15"/>
+      <c r="B247" s="15"/>
+      <c r="C247" s="15"/>
+      <c r="D247" s="15"/>
+      <c r="E247" s="15"/>
+      <c r="F247" s="15"/>
+    </row>
+    <row r="248" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A248" s="15"/>
+      <c r="B248" s="15"/>
+      <c r="C248" s="15"/>
+      <c r="D248" s="15"/>
+      <c r="E248" s="15"/>
+      <c r="F248" s="15"/>
+    </row>
+    <row r="249" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A249" s="15"/>
+      <c r="B249" s="15"/>
+      <c r="C249" s="15"/>
+      <c r="D249" s="15"/>
+      <c r="E249" s="15"/>
+      <c r="F249" s="15"/>
+    </row>
+    <row r="250" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A250" s="15"/>
+      <c r="B250" s="15"/>
+      <c r="C250" s="15"/>
+      <c r="D250" s="15"/>
+      <c r="E250" s="15"/>
+      <c r="F250" s="15"/>
+    </row>
+    <row r="251" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A251" s="15"/>
+      <c r="B251" s="15"/>
+      <c r="C251" s="15"/>
+      <c r="D251" s="15"/>
+      <c r="E251" s="15"/>
+      <c r="F251" s="15"/>
+    </row>
+    <row r="252" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A252" s="15"/>
+      <c r="B252" s="15"/>
+      <c r="C252" s="15"/>
+      <c r="D252" s="15"/>
+      <c r="E252" s="15"/>
+      <c r="F252" s="15"/>
+    </row>
+    <row r="253" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A253" s="15"/>
+      <c r="B253" s="15"/>
+      <c r="C253" s="15"/>
+      <c r="D253" s="15"/>
+      <c r="E253" s="15"/>
+      <c r="F253" s="15"/>
+    </row>
+    <row r="254" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A254" s="15"/>
+      <c r="B254" s="15"/>
+      <c r="C254" s="15"/>
+      <c r="D254" s="15"/>
+      <c r="E254" s="15"/>
+      <c r="F254" s="15"/>
+    </row>
+    <row r="255" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A255" s="15"/>
+      <c r="B255" s="15"/>
+      <c r="C255" s="15"/>
+      <c r="D255" s="15"/>
+      <c r="E255" s="15"/>
+      <c r="F255" s="15"/>
+    </row>
+    <row r="256" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A256" s="15"/>
+      <c r="B256" s="15"/>
+      <c r="C256" s="15"/>
+      <c r="D256" s="15"/>
+      <c r="E256" s="15"/>
+      <c r="F256" s="15"/>
+    </row>
+    <row r="257" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A257" s="15"/>
+      <c r="B257" s="15"/>
+      <c r="C257" s="15"/>
+      <c r="D257" s="15"/>
+      <c r="E257" s="15"/>
+      <c r="F257" s="15"/>
+    </row>
+    <row r="258" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A258" s="15"/>
+      <c r="B258" s="15"/>
+      <c r="C258" s="15"/>
+      <c r="D258" s="15"/>
+      <c r="E258" s="15"/>
+      <c r="F258" s="15"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>